<commit_message>
Planner : tableau Excel nommé TachesVOOMNET + fiche rapide 2 pages
</commit_message>
<xml_diff>
--- a/docs/planner/VOOMNET-planner.xlsx
+++ b/docs/planner/VOOMNET-planner.xlsx
@@ -11,6 +11,7 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Coller Livré" sheetId="2" state="visible" r:id="rId2"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Coller En cours" sheetId="3" state="visible" r:id="rId3"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Coller Planifié" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Taches" sheetId="5" state="visible" r:id="rId5"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -97,7 +98,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="12">
+  <cellXfs count="13">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
@@ -112,6 +113,7 @@
     <xf numFmtId="0" fontId="4" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="6" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="7" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="3" fillId="2" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -186,6 +188,23 @@
     </indexedColors>
   </colors>
 </styleSheet>
+</file>
+
+<file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="TachesVOOMNET" displayName="TachesVOOMNET" ref="A1:H45" headerRowCount="1">
+  <autoFilter ref="A1:H45"/>
+  <tableColumns count="8">
+    <tableColumn id="1" name="Module"/>
+    <tableColumn id="2" name="Tache"/>
+    <tableColumn id="3" name="Compartiment"/>
+    <tableColumn id="4" name="Avancement"/>
+    <tableColumn id="5" name="Echeance"/>
+    <tableColumn id="6" name="Priorite"/>
+    <tableColumn id="7" name="Responsable"/>
+    <tableColumn id="8" name="Notes"/>
+  </tableColumns>
+  <tableStyleInfo name="TableStyleMedium12" showRowStripes="1"/>
+</table>
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
@@ -3135,4 +3154,1833 @@
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:H45"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="16" customWidth="1" min="1" max="1"/>
+    <col width="58" customWidth="1" min="2" max="2"/>
+    <col width="15" customWidth="1" min="3" max="3"/>
+    <col width="13" customWidth="1" min="4" max="4"/>
+    <col width="12" customWidth="1" min="5" max="5"/>
+    <col width="10" customWidth="1" min="6" max="6"/>
+    <col width="13" customWidth="1" min="7" max="7"/>
+    <col width="46" customWidth="1" min="8" max="8"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="12" t="inlineStr">
+        <is>
+          <t>Module</t>
+        </is>
+      </c>
+      <c r="B1" s="12" t="inlineStr">
+        <is>
+          <t>Tache</t>
+        </is>
+      </c>
+      <c r="C1" s="12" t="inlineStr">
+        <is>
+          <t>Compartiment</t>
+        </is>
+      </c>
+      <c r="D1" s="12" t="inlineStr">
+        <is>
+          <t>Avancement</t>
+        </is>
+      </c>
+      <c r="E1" s="12" t="inlineStr">
+        <is>
+          <t>Echeance</t>
+        </is>
+      </c>
+      <c r="F1" s="12" t="inlineStr">
+        <is>
+          <t>Priorite</t>
+        </is>
+      </c>
+      <c r="G1" s="12" t="inlineStr">
+        <is>
+          <t>Responsable</t>
+        </is>
+      </c>
+      <c r="H1" s="12" t="inlineStr">
+        <is>
+          <t>Notes</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>Cadrage</t>
+        </is>
+      </c>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>Cadrage et analyse des besoins</t>
+        </is>
+      </c>
+      <c r="C2" t="inlineStr">
+        <is>
+          <t>Livré</t>
+        </is>
+      </c>
+      <c r="D2" t="n">
+        <v>100</v>
+      </c>
+      <c r="E2" t="inlineStr">
+        <is>
+          <t>28/08/2026</t>
+        </is>
+      </c>
+      <c r="F2" t="inlineStr">
+        <is>
+          <t>Haute</t>
+        </is>
+      </c>
+      <c r="G2" t="inlineStr">
+        <is>
+          <t>Projet</t>
+        </is>
+      </c>
+      <c r="H2" t="inlineStr">
+        <is>
+          <t>Objectifs, périmètre, règles de gestion</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>Cadrage</t>
+        </is>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>Choix de l'architecture (Next.js + Supabase)</t>
+        </is>
+      </c>
+      <c r="C3" t="inlineStr">
+        <is>
+          <t>Livré</t>
+        </is>
+      </c>
+      <c r="D3" t="n">
+        <v>100</v>
+      </c>
+      <c r="E3" t="inlineStr">
+        <is>
+          <t>28/08/2026</t>
+        </is>
+      </c>
+      <c r="F3" t="inlineStr">
+        <is>
+          <t>Haute</t>
+        </is>
+      </c>
+      <c r="G3" t="inlineStr">
+        <is>
+          <t>DSI</t>
+        </is>
+      </c>
+      <c r="H3" t="inlineStr">
+        <is>
+          <t>Application web + base temps réel</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>Sécurité</t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>Authentification et gestion des 3 rôles</t>
+        </is>
+      </c>
+      <c r="C4" t="inlineStr">
+        <is>
+          <t>Livré</t>
+        </is>
+      </c>
+      <c r="D4" t="n">
+        <v>100</v>
+      </c>
+      <c r="E4" t="inlineStr">
+        <is>
+          <t>29/08/2026</t>
+        </is>
+      </c>
+      <c r="F4" t="inlineStr">
+        <is>
+          <t>Haute</t>
+        </is>
+      </c>
+      <c r="G4" t="inlineStr">
+        <is>
+          <t>DSI</t>
+        </is>
+      </c>
+      <c r="H4" t="inlineStr">
+        <is>
+          <t>Demandeur / Responsable / Administrateur</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>Demandes</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>Module demandes d'achat (assistant 6 étapes)</t>
+        </is>
+      </c>
+      <c r="C5" t="inlineStr">
+        <is>
+          <t>Livré</t>
+        </is>
+      </c>
+      <c r="D5" t="n">
+        <v>100</v>
+      </c>
+      <c r="E5" t="inlineStr">
+        <is>
+          <t>29/08/2026</t>
+        </is>
+      </c>
+      <c r="F5" t="inlineStr">
+        <is>
+          <t>Haute</t>
+        </is>
+      </c>
+      <c r="G5" t="inlineStr">
+        <is>
+          <t>DSI</t>
+        </is>
+      </c>
+      <c r="H5" t="inlineStr">
+        <is>
+          <t>Création, brouillon, reprise</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>Demandes</t>
+        </is>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>Numérotation automatique ACH-AAAA-NNNNN</t>
+        </is>
+      </c>
+      <c r="C6" t="inlineStr">
+        <is>
+          <t>Livré</t>
+        </is>
+      </c>
+      <c r="D6" t="n">
+        <v>100</v>
+      </c>
+      <c r="E6" t="inlineStr">
+        <is>
+          <t>29/08/2026</t>
+        </is>
+      </c>
+      <c r="F6" t="inlineStr">
+        <is>
+          <t>Haute</t>
+        </is>
+      </c>
+      <c r="G6" t="inlineStr">
+        <is>
+          <t>DSI</t>
+        </is>
+      </c>
+      <c r="H6" t="inlineStr">
+        <is>
+          <t>Compteur partagé, sans doublon</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>Demandes</t>
+        </is>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>Rendre le coût présumé facultatif</t>
+        </is>
+      </c>
+      <c r="C7" t="inlineStr">
+        <is>
+          <t>Livré</t>
+        </is>
+      </c>
+      <c r="D7" t="n">
+        <v>100</v>
+      </c>
+      <c r="E7" t="inlineStr">
+        <is>
+          <t>01/09/2026</t>
+        </is>
+      </c>
+      <c r="F7" t="inlineStr">
+        <is>
+          <t>Moyenne</t>
+        </is>
+      </c>
+      <c r="G7" t="inlineStr">
+        <is>
+          <t>DSI</t>
+        </is>
+      </c>
+      <c r="H7" t="inlineStr">
+        <is>
+          <t>Demande créable sans montant</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>Fournisseurs</t>
+        </is>
+      </c>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>Catalogue fournisseurs (création, modification, statut)</t>
+        </is>
+      </c>
+      <c r="C8" t="inlineStr">
+        <is>
+          <t>Livré</t>
+        </is>
+      </c>
+      <c r="D8" t="n">
+        <v>100</v>
+      </c>
+      <c r="E8" t="inlineStr">
+        <is>
+          <t>30/08/2026</t>
+        </is>
+      </c>
+      <c r="F8" t="inlineStr">
+        <is>
+          <t>Haute</t>
+        </is>
+      </c>
+      <c r="G8" t="inlineStr">
+        <is>
+          <t>DSI</t>
+        </is>
+      </c>
+      <c r="H8" t="inlineStr">
+        <is>
+          <t>Nom, références, emplacement, WhatsApp, site</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>Fournisseurs</t>
+        </is>
+      </c>
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>Import des fournisseurs (Excel, CSV, JSON)</t>
+        </is>
+      </c>
+      <c r="C9" t="inlineStr">
+        <is>
+          <t>Livré</t>
+        </is>
+      </c>
+      <c r="D9" t="n">
+        <v>100</v>
+      </c>
+      <c r="E9" t="inlineStr">
+        <is>
+          <t>30/08/2026</t>
+        </is>
+      </c>
+      <c r="F9" t="inlineStr">
+        <is>
+          <t>Haute</t>
+        </is>
+      </c>
+      <c r="G9" t="inlineStr">
+        <is>
+          <t>DSI</t>
+        </is>
+      </c>
+      <c r="H9" t="inlineStr">
+        <is>
+          <t>Aperçu, lignes invalides signalées</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>Fournisseurs</t>
+        </is>
+      </c>
+      <c r="B10" t="inlineStr">
+        <is>
+          <t>Export des fournisseurs et modèles de fichiers</t>
+        </is>
+      </c>
+      <c r="C10" t="inlineStr">
+        <is>
+          <t>Livré</t>
+        </is>
+      </c>
+      <c r="D10" t="n">
+        <v>100</v>
+      </c>
+      <c r="E10" t="inlineStr">
+        <is>
+          <t>30/08/2026</t>
+        </is>
+      </c>
+      <c r="F10" t="inlineStr">
+        <is>
+          <t>Moyenne</t>
+        </is>
+      </c>
+      <c r="G10" t="inlineStr">
+        <is>
+          <t>DSI</t>
+        </is>
+      </c>
+      <c r="H10" t="inlineStr">
+        <is>
+          <t>Excel, JSON, CSV</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>Négociation</t>
+        </is>
+      </c>
+      <c r="B11" t="inlineStr">
+        <is>
+          <t>Grille de négociation article × fournisseur</t>
+        </is>
+      </c>
+      <c r="C11" t="inlineStr">
+        <is>
+          <t>Livré</t>
+        </is>
+      </c>
+      <c r="D11" t="n">
+        <v>100</v>
+      </c>
+      <c r="E11" t="inlineStr">
+        <is>
+          <t>31/08/2026</t>
+        </is>
+      </c>
+      <c r="F11" t="inlineStr">
+        <is>
+          <t>Haute</t>
+        </is>
+      </c>
+      <c r="G11" t="inlineStr">
+        <is>
+          <t>DSI</t>
+        </is>
+      </c>
+      <c r="H11" t="inlineStr">
+        <is>
+          <t>Un prix par article et par fournisseur</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="inlineStr">
+        <is>
+          <t>Négociation</t>
+        </is>
+      </c>
+      <c r="B12" t="inlineStr">
+        <is>
+          <t>Rendre les prix facultatifs (seuil paramétrable)</t>
+        </is>
+      </c>
+      <c r="C12" t="inlineStr">
+        <is>
+          <t>Livré</t>
+        </is>
+      </c>
+      <c r="D12" t="n">
+        <v>100</v>
+      </c>
+      <c r="E12" t="inlineStr">
+        <is>
+          <t>02/09/2026</t>
+        </is>
+      </c>
+      <c r="F12" t="inlineStr">
+        <is>
+          <t>Haute</t>
+        </is>
+      </c>
+      <c r="G12" t="inlineStr">
+        <is>
+          <t>DSI</t>
+        </is>
+      </c>
+      <c r="H12" t="inlineStr">
+        <is>
+          <t>Seuil 0 = facultatif</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="inlineStr">
+        <is>
+          <t>Négociation</t>
+        </is>
+      </c>
+      <c r="B13" t="inlineStr">
+        <is>
+          <t>Coût total rendu (remise, TVA, frais de livraison)</t>
+        </is>
+      </c>
+      <c r="C13" t="inlineStr">
+        <is>
+          <t>Livré</t>
+        </is>
+      </c>
+      <c r="D13" t="n">
+        <v>100</v>
+      </c>
+      <c r="E13" t="inlineStr">
+        <is>
+          <t>31/08/2026</t>
+        </is>
+      </c>
+      <c r="F13" t="inlineStr">
+        <is>
+          <t>Haute</t>
+        </is>
+      </c>
+      <c r="G13" t="inlineStr">
+        <is>
+          <t>DSI</t>
+        </is>
+      </c>
+      <c r="H13" t="inlineStr">
+        <is>
+          <t>Comparaison fiable des offres</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="inlineStr">
+        <is>
+          <t>Comparaison</t>
+        </is>
+      </c>
+      <c r="B14" t="inlineStr">
+        <is>
+          <t>Score multicritère /100 et classement</t>
+        </is>
+      </c>
+      <c r="C14" t="inlineStr">
+        <is>
+          <t>Livré</t>
+        </is>
+      </c>
+      <c r="D14" t="n">
+        <v>100</v>
+      </c>
+      <c r="E14" t="inlineStr">
+        <is>
+          <t>31/08/2026</t>
+        </is>
+      </c>
+      <c r="F14" t="inlineStr">
+        <is>
+          <t>Moyenne</t>
+        </is>
+      </c>
+      <c r="G14" t="inlineStr">
+        <is>
+          <t>DSI</t>
+        </is>
+      </c>
+      <c r="H14" t="inlineStr">
+        <is>
+          <t>Prix, délai, garantie, paiement</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="inlineStr">
+        <is>
+          <t>Comparaison</t>
+        </is>
+      </c>
+      <c r="B15" t="inlineStr">
+        <is>
+          <t>Tableau croisé et meilleurs prix surlignés</t>
+        </is>
+      </c>
+      <c r="C15" t="inlineStr">
+        <is>
+          <t>Livré</t>
+        </is>
+      </c>
+      <c r="D15" t="n">
+        <v>100</v>
+      </c>
+      <c r="E15" t="inlineStr">
+        <is>
+          <t>31/08/2026</t>
+        </is>
+      </c>
+      <c r="F15" t="inlineStr">
+        <is>
+          <t>Haute</t>
+        </is>
+      </c>
+      <c r="G15" t="inlineStr">
+        <is>
+          <t>DSI</t>
+        </is>
+      </c>
+      <c r="H15" t="inlineStr">
+        <is>
+          <t>Lecture seule, étape non bloquante</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="inlineStr">
+        <is>
+          <t>Validation</t>
+        </is>
+      </c>
+      <c r="B16" t="inlineStr">
+        <is>
+          <t>Circuit de validation (approuver / refuser / modifier)</t>
+        </is>
+      </c>
+      <c r="C16" t="inlineStr">
+        <is>
+          <t>Livré</t>
+        </is>
+      </c>
+      <c r="D16" t="n">
+        <v>100</v>
+      </c>
+      <c r="E16" t="inlineStr">
+        <is>
+          <t>01/09/2026</t>
+        </is>
+      </c>
+      <c r="F16" t="inlineStr">
+        <is>
+          <t>Haute</t>
+        </is>
+      </c>
+      <c r="G16" t="inlineStr">
+        <is>
+          <t>DSI</t>
+        </is>
+      </c>
+      <c r="H16" t="inlineStr">
+        <is>
+          <t>Motif obligatoire si refus</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="inlineStr">
+        <is>
+          <t>Commandes</t>
+        </is>
+      </c>
+      <c r="B17" t="inlineStr">
+        <is>
+          <t>Bons de commande BC-AAAA-NNNNN et confirmation</t>
+        </is>
+      </c>
+      <c r="C17" t="inlineStr">
+        <is>
+          <t>Livré</t>
+        </is>
+      </c>
+      <c r="D17" t="n">
+        <v>100</v>
+      </c>
+      <c r="E17" t="inlineStr">
+        <is>
+          <t>01/09/2026</t>
+        </is>
+      </c>
+      <c r="F17" t="inlineStr">
+        <is>
+          <t>Haute</t>
+        </is>
+      </c>
+      <c r="G17" t="inlineStr">
+        <is>
+          <t>DSI</t>
+        </is>
+      </c>
+      <c r="H17" t="inlineStr">
+        <is>
+          <t>Lignes aux prix négociés</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" t="inlineStr">
+        <is>
+          <t>Commandes</t>
+        </is>
+      </c>
+      <c r="B18" t="inlineStr">
+        <is>
+          <t>Commande et impression sans fournisseur ni prix</t>
+        </is>
+      </c>
+      <c r="C18" t="inlineStr">
+        <is>
+          <t>Livré</t>
+        </is>
+      </c>
+      <c r="D18" t="n">
+        <v>100</v>
+      </c>
+      <c r="E18" t="inlineStr">
+        <is>
+          <t>02/09/2026</t>
+        </is>
+      </c>
+      <c r="F18" t="inlineStr">
+        <is>
+          <t>Moyenne</t>
+        </is>
+      </c>
+      <c r="G18" t="inlineStr">
+        <is>
+          <t>DSI</t>
+        </is>
+      </c>
+      <c r="H18" t="inlineStr">
+        <is>
+          <t>Cas des consultations en cours</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" t="inlineStr">
+        <is>
+          <t>Réceptions</t>
+        </is>
+      </c>
+      <c r="B19" t="inlineStr">
+        <is>
+          <t>Réceptions complètes et partielles</t>
+        </is>
+      </c>
+      <c r="C19" t="inlineStr">
+        <is>
+          <t>Livré</t>
+        </is>
+      </c>
+      <c r="D19" t="n">
+        <v>100</v>
+      </c>
+      <c r="E19" t="inlineStr">
+        <is>
+          <t>01/09/2026</t>
+        </is>
+      </c>
+      <c r="F19" t="inlineStr">
+        <is>
+          <t>Haute</t>
+        </is>
+      </c>
+      <c r="G19" t="inlineStr">
+        <is>
+          <t>DSI</t>
+        </is>
+      </c>
+      <c r="H19" t="inlineStr">
+        <is>
+          <t>Clôture automatique si complète</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" t="inlineStr">
+        <is>
+          <t>Administration</t>
+        </is>
+      </c>
+      <c r="B20" t="inlineStr">
+        <is>
+          <t>Suppressions (demande, commande, réception, utilisateur)</t>
+        </is>
+      </c>
+      <c r="C20" t="inlineStr">
+        <is>
+          <t>Livré</t>
+        </is>
+      </c>
+      <c r="D20" t="n">
+        <v>100</v>
+      </c>
+      <c r="E20" t="inlineStr">
+        <is>
+          <t>01/09/2026</t>
+        </is>
+      </c>
+      <c r="F20" t="inlineStr">
+        <is>
+          <t>Haute</t>
+        </is>
+      </c>
+      <c r="G20" t="inlineStr">
+        <is>
+          <t>DSI</t>
+        </is>
+      </c>
+      <c r="H20" t="inlineStr">
+        <is>
+          <t>Cascades et garde-fous</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" t="inlineStr">
+        <is>
+          <t>Alertes</t>
+        </is>
+      </c>
+      <c r="B21" t="inlineStr">
+        <is>
+          <t>Notifications et relances automatiques</t>
+        </is>
+      </c>
+      <c r="C21" t="inlineStr">
+        <is>
+          <t>Livré</t>
+        </is>
+      </c>
+      <c r="D21" t="n">
+        <v>100</v>
+      </c>
+      <c r="E21" t="inlineStr">
+        <is>
+          <t>02/09/2026</t>
+        </is>
+      </c>
+      <c r="F21" t="inlineStr">
+        <is>
+          <t>Haute</t>
+        </is>
+      </c>
+      <c r="G21" t="inlineStr">
+        <is>
+          <t>DSI</t>
+        </is>
+      </c>
+      <c r="H21" t="inlineStr">
+        <is>
+          <t>Validation et réception, anti-doublon</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" t="inlineStr">
+        <is>
+          <t>Alertes</t>
+        </is>
+      </c>
+      <c r="B22" t="inlineStr">
+        <is>
+          <t>Bandeau d'alertes et pastilles sur le tableau de bord</t>
+        </is>
+      </c>
+      <c r="C22" t="inlineStr">
+        <is>
+          <t>Livré</t>
+        </is>
+      </c>
+      <c r="D22" t="n">
+        <v>100</v>
+      </c>
+      <c r="E22" t="inlineStr">
+        <is>
+          <t>02/09/2026</t>
+        </is>
+      </c>
+      <c r="F22" t="inlineStr">
+        <is>
+          <t>Moyenne</t>
+        </is>
+      </c>
+      <c r="G22" t="inlineStr">
+        <is>
+          <t>DSI</t>
+        </is>
+      </c>
+      <c r="H22" t="inlineStr">
+        <is>
+          <t>Vue immédiate des retards</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" t="inlineStr">
+        <is>
+          <t>Alertes</t>
+        </is>
+      </c>
+      <c r="B23" t="inlineStr">
+        <is>
+          <t>Sons de notification (3 niveaux) et volume réglable</t>
+        </is>
+      </c>
+      <c r="C23" t="inlineStr">
+        <is>
+          <t>Livré</t>
+        </is>
+      </c>
+      <c r="D23" t="n">
+        <v>100</v>
+      </c>
+      <c r="E23" t="inlineStr">
+        <is>
+          <t>02/09/2026</t>
+        </is>
+      </c>
+      <c r="F23" t="inlineStr">
+        <is>
+          <t>Moyenne</t>
+        </is>
+      </c>
+      <c r="G23" t="inlineStr">
+        <is>
+          <t>DSI</t>
+        </is>
+      </c>
+      <c r="H23" t="inlineStr">
+        <is>
+          <t>Avec son de secours si bloqué</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" t="inlineStr">
+        <is>
+          <t>Alertes</t>
+        </is>
+      </c>
+      <c r="B24" t="inlineStr">
+        <is>
+          <t>Alarme répétée jusqu'à lecture du message</t>
+        </is>
+      </c>
+      <c r="C24" t="inlineStr">
+        <is>
+          <t>Livré</t>
+        </is>
+      </c>
+      <c r="D24" t="n">
+        <v>100</v>
+      </c>
+      <c r="E24" t="inlineStr">
+        <is>
+          <t>02/09/2026</t>
+        </is>
+      </c>
+      <c r="F24" t="inlineStr">
+        <is>
+          <t>Moyenne</t>
+        </is>
+      </c>
+      <c r="G24" t="inlineStr">
+        <is>
+          <t>DSI</t>
+        </is>
+      </c>
+      <c r="H24" t="inlineStr">
+        <is>
+          <t>15 s, maximum 10 répétitions</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" t="inlineStr">
+        <is>
+          <t>Alertes</t>
+        </is>
+      </c>
+      <c r="B25" t="inlineStr">
+        <is>
+          <t>Notifications du navigateur (bulles système)</t>
+        </is>
+      </c>
+      <c r="C25" t="inlineStr">
+        <is>
+          <t>Livré</t>
+        </is>
+      </c>
+      <c r="D25" t="n">
+        <v>100</v>
+      </c>
+      <c r="E25" t="inlineStr">
+        <is>
+          <t>02/09/2026</t>
+        </is>
+      </c>
+      <c r="F25" t="inlineStr">
+        <is>
+          <t>Moyenne</t>
+        </is>
+      </c>
+      <c r="G25" t="inlineStr">
+        <is>
+          <t>DSI</t>
+        </is>
+      </c>
+      <c r="H25" t="inlineStr">
+        <is>
+          <t>Actives onglet en arrière-plan</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" t="inlineStr">
+        <is>
+          <t>Alertes</t>
+        </is>
+      </c>
+      <c r="B26" t="inlineStr">
+        <is>
+          <t>Alerte visuelle (onglet clignotant, pastille pulsante)</t>
+        </is>
+      </c>
+      <c r="C26" t="inlineStr">
+        <is>
+          <t>Livré</t>
+        </is>
+      </c>
+      <c r="D26" t="n">
+        <v>100</v>
+      </c>
+      <c r="E26" t="inlineStr">
+        <is>
+          <t>02/09/2026</t>
+        </is>
+      </c>
+      <c r="F26" t="inlineStr">
+        <is>
+          <t>Moyenne</t>
+        </is>
+      </c>
+      <c r="G26" t="inlineStr">
+        <is>
+          <t>DSI</t>
+        </is>
+      </c>
+      <c r="H26" t="inlineStr">
+        <is>
+          <t>Secours si le son est coupé</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" t="inlineStr">
+        <is>
+          <t>Documents</t>
+        </is>
+      </c>
+      <c r="B27" t="inlineStr">
+        <is>
+          <t>Impression fiche de demande et bon de commande</t>
+        </is>
+      </c>
+      <c r="C27" t="inlineStr">
+        <is>
+          <t>Livré</t>
+        </is>
+      </c>
+      <c r="D27" t="n">
+        <v>100</v>
+      </c>
+      <c r="E27" t="inlineStr">
+        <is>
+          <t>02/09/2026</t>
+        </is>
+      </c>
+      <c r="F27" t="inlineStr">
+        <is>
+          <t>Haute</t>
+        </is>
+      </c>
+      <c r="G27" t="inlineStr">
+        <is>
+          <t>DSI</t>
+        </is>
+      </c>
+      <c r="H27" t="inlineStr">
+        <is>
+          <t>Colonnes de prix vides à compléter</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" t="inlineStr">
+        <is>
+          <t>Documents</t>
+        </is>
+      </c>
+      <c r="B28" t="inlineStr">
+        <is>
+          <t>Exports PDF (demandes, commandes, réceptions)</t>
+        </is>
+      </c>
+      <c r="C28" t="inlineStr">
+        <is>
+          <t>Livré</t>
+        </is>
+      </c>
+      <c r="D28" t="n">
+        <v>100</v>
+      </c>
+      <c r="E28" t="inlineStr">
+        <is>
+          <t>01/09/2026</t>
+        </is>
+      </c>
+      <c r="F28" t="inlineStr">
+        <is>
+          <t>Haute</t>
+        </is>
+      </c>
+      <c r="G28" t="inlineStr">
+        <is>
+          <t>DSI</t>
+        </is>
+      </c>
+      <c r="H28" t="inlineStr">
+        <is>
+          <t>jsPDF, repli impression</t>
+        </is>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" t="inlineStr">
+        <is>
+          <t>Documents</t>
+        </is>
+      </c>
+      <c r="B29" t="inlineStr">
+        <is>
+          <t>Exports Excel et CSV</t>
+        </is>
+      </c>
+      <c r="C29" t="inlineStr">
+        <is>
+          <t>Livré</t>
+        </is>
+      </c>
+      <c r="D29" t="n">
+        <v>100</v>
+      </c>
+      <c r="E29" t="inlineStr">
+        <is>
+          <t>01/09/2026</t>
+        </is>
+      </c>
+      <c r="F29" t="inlineStr">
+        <is>
+          <t>Moyenne</t>
+        </is>
+      </c>
+      <c r="G29" t="inlineStr">
+        <is>
+          <t>DSI</t>
+        </is>
+      </c>
+      <c r="H29" t="inlineStr">
+        <is>
+          <t>Comparaison incluse</t>
+        </is>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" t="inlineStr">
+        <is>
+          <t>Identité</t>
+        </is>
+      </c>
+      <c r="B30" t="inlineStr">
+        <is>
+          <t>Intégration du logo et charte violet / bleu nuit</t>
+        </is>
+      </c>
+      <c r="C30" t="inlineStr">
+        <is>
+          <t>Livré</t>
+        </is>
+      </c>
+      <c r="D30" t="n">
+        <v>100</v>
+      </c>
+      <c r="E30" t="inlineStr">
+        <is>
+          <t>02/09/2026</t>
+        </is>
+      </c>
+      <c r="F30" t="inlineStr">
+        <is>
+          <t>Moyenne</t>
+        </is>
+      </c>
+      <c r="G30" t="inlineStr">
+        <is>
+          <t>Direction</t>
+        </is>
+      </c>
+      <c r="H30" t="inlineStr">
+        <is>
+          <t>Site, impressions, PDF, favicon</t>
+        </is>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" t="inlineStr">
+        <is>
+          <t>Données</t>
+        </is>
+      </c>
+      <c r="B31" t="inlineStr">
+        <is>
+          <t>Synchronisation Supabase en temps réel</t>
+        </is>
+      </c>
+      <c r="C31" t="inlineStr">
+        <is>
+          <t>Livré</t>
+        </is>
+      </c>
+      <c r="D31" t="n">
+        <v>100</v>
+      </c>
+      <c r="E31" t="inlineStr">
+        <is>
+          <t>02/09/2026</t>
+        </is>
+      </c>
+      <c r="F31" t="inlineStr">
+        <is>
+          <t>Haute</t>
+        </is>
+      </c>
+      <c r="G31" t="inlineStr">
+        <is>
+          <t>DSI</t>
+        </is>
+      </c>
+      <c r="H31" t="inlineStr">
+        <is>
+          <t>Partage entre tous les postes</t>
+        </is>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" t="inlineStr">
+        <is>
+          <t>Données</t>
+        </is>
+      </c>
+      <c r="B32" t="inlineStr">
+        <is>
+          <t>Sécurisation anti-écrasement entre appareils</t>
+        </is>
+      </c>
+      <c r="C32" t="inlineStr">
+        <is>
+          <t>Livré</t>
+        </is>
+      </c>
+      <c r="D32" t="n">
+        <v>100</v>
+      </c>
+      <c r="E32" t="inlineStr">
+        <is>
+          <t>02/09/2026</t>
+        </is>
+      </c>
+      <c r="F32" t="inlineStr">
+        <is>
+          <t>Haute</t>
+        </is>
+      </c>
+      <c r="G32" t="inlineStr">
+        <is>
+          <t>DSI</t>
+        </is>
+      </c>
+      <c r="H32" t="inlineStr">
+        <is>
+          <t>Le serveur fait foi au démarrage</t>
+        </is>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" t="inlineStr">
+        <is>
+          <t>Pilotage</t>
+        </is>
+      </c>
+      <c r="B33" t="inlineStr">
+        <is>
+          <t>Tableau de bord graphique (3 graphiques)</t>
+        </is>
+      </c>
+      <c r="C33" t="inlineStr">
+        <is>
+          <t>Livré</t>
+        </is>
+      </c>
+      <c r="D33" t="n">
+        <v>100</v>
+      </c>
+      <c r="E33" t="inlineStr">
+        <is>
+          <t>02/09/2026</t>
+        </is>
+      </c>
+      <c r="F33" t="inlineStr">
+        <is>
+          <t>Moyenne</t>
+        </is>
+      </c>
+      <c r="G33" t="inlineStr">
+        <is>
+          <t>DSI</t>
+        </is>
+      </c>
+      <c r="H33" t="inlineStr">
+        <is>
+          <t>Achats 12 mois, répartition, top 5</t>
+        </is>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" t="inlineStr">
+        <is>
+          <t>Qualité</t>
+        </is>
+      </c>
+      <c r="B34" t="inlineStr">
+        <is>
+          <t>Suite de tests automatisés (197 contrôles)</t>
+        </is>
+      </c>
+      <c r="C34" t="inlineStr">
+        <is>
+          <t>Livré</t>
+        </is>
+      </c>
+      <c r="D34" t="n">
+        <v>100</v>
+      </c>
+      <c r="E34" t="inlineStr">
+        <is>
+          <t>02/09/2026</t>
+        </is>
+      </c>
+      <c r="F34" t="inlineStr">
+        <is>
+          <t>Haute</t>
+        </is>
+      </c>
+      <c r="G34" t="inlineStr">
+        <is>
+          <t>DSI</t>
+        </is>
+      </c>
+      <c r="H34" t="inlineStr">
+        <is>
+          <t>13 séries, exécutées avant publication</t>
+        </is>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" t="inlineStr">
+        <is>
+          <t>Déploiement</t>
+        </is>
+      </c>
+      <c r="B35" t="inlineStr">
+        <is>
+          <t>Déploiement continu GitHub vers Vercel</t>
+        </is>
+      </c>
+      <c r="C35" t="inlineStr">
+        <is>
+          <t>Livré</t>
+        </is>
+      </c>
+      <c r="D35" t="n">
+        <v>100</v>
+      </c>
+      <c r="E35" t="inlineStr">
+        <is>
+          <t>02/09/2026</t>
+        </is>
+      </c>
+      <c r="F35" t="inlineStr">
+        <is>
+          <t>Haute</t>
+        </is>
+      </c>
+      <c r="G35" t="inlineStr">
+        <is>
+          <t>DSI</t>
+        </is>
+      </c>
+      <c r="H35" t="inlineStr">
+        <is>
+          <t>Une commande : scripts/publish.mjs</t>
+        </is>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" t="inlineStr">
+        <is>
+          <t>Documentation</t>
+        </is>
+      </c>
+      <c r="B36" t="inlineStr">
+        <is>
+          <t>Cahier des charges et synthèse direction</t>
+        </is>
+      </c>
+      <c r="C36" t="inlineStr">
+        <is>
+          <t>Livré</t>
+        </is>
+      </c>
+      <c r="D36" t="n">
+        <v>100</v>
+      </c>
+      <c r="E36" t="inlineStr">
+        <is>
+          <t>02/09/2026</t>
+        </is>
+      </c>
+      <c r="F36" t="inlineStr">
+        <is>
+          <t>Moyenne</t>
+        </is>
+      </c>
+      <c r="G36" t="inlineStr">
+        <is>
+          <t>DSI</t>
+        </is>
+      </c>
+      <c r="H36" t="inlineStr">
+        <is>
+          <t>PDF et Word, 14 et 4 pages</t>
+        </is>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" t="inlineStr">
+        <is>
+          <t>Qualité</t>
+        </is>
+      </c>
+      <c r="B37" t="inlineStr">
+        <is>
+          <t>Recette utilisateur et ajustements</t>
+        </is>
+      </c>
+      <c r="C37" t="inlineStr">
+        <is>
+          <t>En cours</t>
+        </is>
+      </c>
+      <c r="D37" t="n">
+        <v>60</v>
+      </c>
+      <c r="E37" t="inlineStr">
+        <is>
+          <t>05/09/2026</t>
+        </is>
+      </c>
+      <c r="F37" t="inlineStr">
+        <is>
+          <t>Haute</t>
+        </is>
+      </c>
+      <c r="G37" t="inlineStr">
+        <is>
+          <t>Direction</t>
+        </is>
+      </c>
+      <c r="H37" t="inlineStr">
+        <is>
+          <t>Retours des utilisateurs finaux</t>
+        </is>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" t="inlineStr">
+        <is>
+          <t>Sécurité</t>
+        </is>
+      </c>
+      <c r="B38" t="inlineStr">
+        <is>
+          <t>Durcissement des politiques d'accès (RLS)</t>
+        </is>
+      </c>
+      <c r="C38" t="inlineStr">
+        <is>
+          <t>En cours</t>
+        </is>
+      </c>
+      <c r="D38" t="n">
+        <v>30</v>
+      </c>
+      <c r="E38" t="inlineStr">
+        <is>
+          <t>09/09/2026</t>
+        </is>
+      </c>
+      <c r="F38" t="inlineStr">
+        <is>
+          <t>Haute</t>
+        </is>
+      </c>
+      <c r="G38" t="inlineStr">
+        <is>
+          <t>DSI</t>
+        </is>
+      </c>
+      <c r="H38" t="inlineStr">
+        <is>
+          <t>Restreindre par rôle avant généralisation</t>
+        </is>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" t="inlineStr">
+        <is>
+          <t>Sécurité</t>
+        </is>
+      </c>
+      <c r="B39" t="inlineStr">
+        <is>
+          <t>Journal d'audit des actions sensibles</t>
+        </is>
+      </c>
+      <c r="C39" t="inlineStr">
+        <is>
+          <t>En cours</t>
+        </is>
+      </c>
+      <c r="D39" t="n">
+        <v>15</v>
+      </c>
+      <c r="E39" t="inlineStr">
+        <is>
+          <t>12/09/2026</t>
+        </is>
+      </c>
+      <c r="F39" t="inlineStr">
+        <is>
+          <t>Haute</t>
+        </is>
+      </c>
+      <c r="G39" t="inlineStr">
+        <is>
+          <t>DSI</t>
+        </is>
+      </c>
+      <c r="H39" t="inlineStr">
+        <is>
+          <t>Qui a supprimé/modifié quoi et quand</t>
+        </is>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" t="inlineStr">
+        <is>
+          <t>Sécurité</t>
+        </is>
+      </c>
+      <c r="B40" t="inlineStr">
+        <is>
+          <t>Authentification sécurisée (mots de passe hachés)</t>
+        </is>
+      </c>
+      <c r="C40" t="inlineStr">
+        <is>
+          <t>Planifié</t>
+        </is>
+      </c>
+      <c r="D40" t="n">
+        <v>0</v>
+      </c>
+      <c r="E40" t="inlineStr">
+        <is>
+          <t>19/09/2026</t>
+        </is>
+      </c>
+      <c r="F40" t="inlineStr">
+        <is>
+          <t>Haute</t>
+        </is>
+      </c>
+      <c r="G40" t="inlineStr">
+        <is>
+          <t>DSI</t>
+        </is>
+      </c>
+      <c r="H40" t="inlineStr">
+        <is>
+          <t>Migration vers Supabase Auth</t>
+        </is>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" t="inlineStr">
+        <is>
+          <t>Alertes</t>
+        </is>
+      </c>
+      <c r="B41" t="inlineStr">
+        <is>
+          <t>Notifications par e-mail</t>
+        </is>
+      </c>
+      <c r="C41" t="inlineStr">
+        <is>
+          <t>Planifié</t>
+        </is>
+      </c>
+      <c r="D41" t="n">
+        <v>0</v>
+      </c>
+      <c r="E41" t="inlineStr">
+        <is>
+          <t>26/09/2026</t>
+        </is>
+      </c>
+      <c r="F41" t="inlineStr">
+        <is>
+          <t>Moyenne</t>
+        </is>
+      </c>
+      <c r="G41" t="inlineStr">
+        <is>
+          <t>DSI</t>
+        </is>
+      </c>
+      <c r="H41" t="inlineStr">
+        <is>
+          <t>Réduction des délais de réponse</t>
+        </is>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" t="inlineStr">
+        <is>
+          <t>Pilotage</t>
+        </is>
+      </c>
+      <c r="B42" t="inlineStr">
+        <is>
+          <t>Budgets par service avec alerte de dépassement</t>
+        </is>
+      </c>
+      <c r="C42" t="inlineStr">
+        <is>
+          <t>Planifié</t>
+        </is>
+      </c>
+      <c r="D42" t="n">
+        <v>0</v>
+      </c>
+      <c r="E42" t="inlineStr">
+        <is>
+          <t>10/10/2026</t>
+        </is>
+      </c>
+      <c r="F42" t="inlineStr">
+        <is>
+          <t>Moyenne</t>
+        </is>
+      </c>
+      <c r="G42" t="inlineStr">
+        <is>
+          <t>Direction</t>
+        </is>
+      </c>
+      <c r="H42" t="inlineStr">
+        <is>
+          <t>Pilotage financier</t>
+        </is>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43" t="inlineStr">
+        <is>
+          <t>Fournisseurs</t>
+        </is>
+      </c>
+      <c r="B43" t="inlineStr">
+        <is>
+          <t>Portail fournisseur (saisie directe des offres)</t>
+        </is>
+      </c>
+      <c r="C43" t="inlineStr">
+        <is>
+          <t>Planifié</t>
+        </is>
+      </c>
+      <c r="D43" t="n">
+        <v>0</v>
+      </c>
+      <c r="E43" t="inlineStr">
+        <is>
+          <t>24/10/2026</t>
+        </is>
+      </c>
+      <c r="F43" t="inlineStr">
+        <is>
+          <t>Basse</t>
+        </is>
+      </c>
+      <c r="G43" t="inlineStr">
+        <is>
+          <t>DSI</t>
+        </is>
+      </c>
+      <c r="H43" t="inlineStr">
+        <is>
+          <t>Productivité sur les consultations</t>
+        </is>
+      </c>
+    </row>
+    <row r="44">
+      <c r="A44" t="inlineStr">
+        <is>
+          <t>Logistique</t>
+        </is>
+      </c>
+      <c r="B44" t="inlineStr">
+        <is>
+          <t>Gestion des stocks liée aux réceptions</t>
+        </is>
+      </c>
+      <c r="C44" t="inlineStr">
+        <is>
+          <t>Planifié</t>
+        </is>
+      </c>
+      <c r="D44" t="n">
+        <v>0</v>
+      </c>
+      <c r="E44" t="inlineStr">
+        <is>
+          <t>31/10/2026</t>
+        </is>
+      </c>
+      <c r="F44" t="inlineStr">
+        <is>
+          <t>Basse</t>
+        </is>
+      </c>
+      <c r="G44" t="inlineStr">
+        <is>
+          <t>Logistique</t>
+        </is>
+      </c>
+      <c r="H44" t="inlineStr">
+        <is>
+          <t>À cadrer</t>
+        </is>
+      </c>
+    </row>
+    <row r="45">
+      <c r="A45" t="inlineStr">
+        <is>
+          <t>Sécurité</t>
+        </is>
+      </c>
+      <c r="B45" t="inlineStr">
+        <is>
+          <t>Authentification unique (SSO)</t>
+        </is>
+      </c>
+      <c r="C45" t="inlineStr">
+        <is>
+          <t>Planifié</t>
+        </is>
+      </c>
+      <c r="D45" t="n">
+        <v>0</v>
+      </c>
+      <c r="E45" t="inlineStr">
+        <is>
+          <t>31/10/2026</t>
+        </is>
+      </c>
+      <c r="F45" t="inlineStr">
+        <is>
+          <t>Basse</t>
+        </is>
+      </c>
+      <c r="G45" t="inlineStr">
+        <is>
+          <t>DSI</t>
+        </is>
+      </c>
+      <c r="H45" t="inlineStr">
+        <is>
+          <t>Confort utilisateur</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+  <tableParts count="1">
+    <tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>
+  </tableParts>
+</worksheet>
 </file>
</xml_diff>

<commit_message>
Planner : export Grille 9 colonnes validé + lecture par vue (Tableau, Graphiques, Planning)
</commit_message>
<xml_diff>
--- a/docs/planner/VOOMNET-planner.xlsx
+++ b/docs/planner/VOOMNET-planner.xlsx
@@ -12,6 +12,7 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Coller En cours" sheetId="3" state="visible" r:id="rId3"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Coller Planifié" sheetId="4" state="visible" r:id="rId4"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Taches" sheetId="5" state="visible" r:id="rId5"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Grille" sheetId="6" state="visible" r:id="rId6"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -202,6 +203,24 @@
     <tableColumn id="6" name="Priorite"/>
     <tableColumn id="7" name="Responsable"/>
     <tableColumn id="8" name="Notes"/>
+  </tableColumns>
+  <tableStyleInfo name="TableStyleMedium12" showRowStripes="1"/>
+</table>
+</file>
+
+<file path=xl/tables/table2.xml><?xml version="1.0" encoding="utf-8"?>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="2" name="GrilleVOOMNET" displayName="GrilleVOOMNET" ref="A1:I45" headerRowCount="1">
+  <autoFilter ref="A1:I45"/>
+  <tableColumns count="9">
+    <tableColumn id="1" name="Nom de la tâche"/>
+    <tableColumn id="2" name="Compartiment"/>
+    <tableColumn id="3" name="Progression"/>
+    <tableColumn id="4" name="Priorité"/>
+    <tableColumn id="5" name="Assigné à"/>
+    <tableColumn id="6" name="Date de début"/>
+    <tableColumn id="7" name="Date d'échéance"/>
+    <tableColumn id="8" name="Étiquettes"/>
+    <tableColumn id="9" name="Description"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium12" showRowStripes="1"/>
 </table>
@@ -4983,4 +5002,2123 @@
     <tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>
   </tableParts>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:I45"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="58" customWidth="1" min="1" max="1"/>
+    <col width="15" customWidth="1" min="2" max="2"/>
+    <col width="14" customWidth="1" min="3" max="3"/>
+    <col width="11" customWidth="1" min="4" max="4"/>
+    <col width="14" customWidth="1" min="5" max="5"/>
+    <col width="13" customWidth="1" min="6" max="6"/>
+    <col width="14" customWidth="1" min="7" max="7"/>
+    <col width="16" customWidth="1" min="8" max="8"/>
+    <col width="46" customWidth="1" min="9" max="9"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="12" t="inlineStr">
+        <is>
+          <t>Nom de la tâche</t>
+        </is>
+      </c>
+      <c r="B1" s="12" t="inlineStr">
+        <is>
+          <t>Compartiment</t>
+        </is>
+      </c>
+      <c r="C1" s="12" t="inlineStr">
+        <is>
+          <t>Progression</t>
+        </is>
+      </c>
+      <c r="D1" s="12" t="inlineStr">
+        <is>
+          <t>Priorité</t>
+        </is>
+      </c>
+      <c r="E1" s="12" t="inlineStr">
+        <is>
+          <t>Assigné à</t>
+        </is>
+      </c>
+      <c r="F1" s="12" t="inlineStr">
+        <is>
+          <t>Date de début</t>
+        </is>
+      </c>
+      <c r="G1" s="12" t="inlineStr">
+        <is>
+          <t>Date d'échéance</t>
+        </is>
+      </c>
+      <c r="H1" s="12" t="inlineStr">
+        <is>
+          <t>Étiquettes</t>
+        </is>
+      </c>
+      <c r="I1" s="12" t="inlineStr">
+        <is>
+          <t>Description</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>[Cadrage] Cadrage et analyse des besoins (100 %)</t>
+        </is>
+      </c>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>Livré</t>
+        </is>
+      </c>
+      <c r="C2" t="inlineStr">
+        <is>
+          <t>Terminé</t>
+        </is>
+      </c>
+      <c r="D2" t="inlineStr">
+        <is>
+          <t>Urgent</t>
+        </is>
+      </c>
+      <c r="E2" t="inlineStr">
+        <is>
+          <t>Projet</t>
+        </is>
+      </c>
+      <c r="F2" t="inlineStr">
+        <is>
+          <t>28/08/2026</t>
+        </is>
+      </c>
+      <c r="G2" t="inlineStr">
+        <is>
+          <t>28/08/2026</t>
+        </is>
+      </c>
+      <c r="H2" t="inlineStr">
+        <is>
+          <t>Cadrage</t>
+        </is>
+      </c>
+      <c r="I2" t="inlineStr">
+        <is>
+          <t>Objectifs, périmètre, règles de gestion</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>[Cadrage] Choix de l'architecture (Next.js + Supabase) (100 %)</t>
+        </is>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>Livré</t>
+        </is>
+      </c>
+      <c r="C3" t="inlineStr">
+        <is>
+          <t>Terminé</t>
+        </is>
+      </c>
+      <c r="D3" t="inlineStr">
+        <is>
+          <t>Urgent</t>
+        </is>
+      </c>
+      <c r="E3" t="inlineStr">
+        <is>
+          <t>DSI</t>
+        </is>
+      </c>
+      <c r="F3" t="inlineStr">
+        <is>
+          <t>28/08/2026</t>
+        </is>
+      </c>
+      <c r="G3" t="inlineStr">
+        <is>
+          <t>28/08/2026</t>
+        </is>
+      </c>
+      <c r="H3" t="inlineStr">
+        <is>
+          <t>Cadrage</t>
+        </is>
+      </c>
+      <c r="I3" t="inlineStr">
+        <is>
+          <t>Application web + base temps réel</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>[Sécurité] Authentification et gestion des 3 rôles (100 %)</t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>Livré</t>
+        </is>
+      </c>
+      <c r="C4" t="inlineStr">
+        <is>
+          <t>Terminé</t>
+        </is>
+      </c>
+      <c r="D4" t="inlineStr">
+        <is>
+          <t>Urgent</t>
+        </is>
+      </c>
+      <c r="E4" t="inlineStr">
+        <is>
+          <t>DSI</t>
+        </is>
+      </c>
+      <c r="F4" t="inlineStr">
+        <is>
+          <t>28/08/2026</t>
+        </is>
+      </c>
+      <c r="G4" t="inlineStr">
+        <is>
+          <t>29/08/2026</t>
+        </is>
+      </c>
+      <c r="H4" t="inlineStr">
+        <is>
+          <t>Sécurité</t>
+        </is>
+      </c>
+      <c r="I4" t="inlineStr">
+        <is>
+          <t>Demandeur / Responsable / Administrateur</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>[Demandes] Module demandes d'achat (assistant 6 étapes) (100 %)</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>Livré</t>
+        </is>
+      </c>
+      <c r="C5" t="inlineStr">
+        <is>
+          <t>Terminé</t>
+        </is>
+      </c>
+      <c r="D5" t="inlineStr">
+        <is>
+          <t>Urgent</t>
+        </is>
+      </c>
+      <c r="E5" t="inlineStr">
+        <is>
+          <t>DSI</t>
+        </is>
+      </c>
+      <c r="F5" t="inlineStr">
+        <is>
+          <t>28/08/2026</t>
+        </is>
+      </c>
+      <c r="G5" t="inlineStr">
+        <is>
+          <t>29/08/2026</t>
+        </is>
+      </c>
+      <c r="H5" t="inlineStr">
+        <is>
+          <t>Demandes</t>
+        </is>
+      </c>
+      <c r="I5" t="inlineStr">
+        <is>
+          <t>Création, brouillon, reprise</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>[Demandes] Numérotation automatique ACH-AAAA-NNNNN (100 %)</t>
+        </is>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>Livré</t>
+        </is>
+      </c>
+      <c r="C6" t="inlineStr">
+        <is>
+          <t>Terminé</t>
+        </is>
+      </c>
+      <c r="D6" t="inlineStr">
+        <is>
+          <t>Urgent</t>
+        </is>
+      </c>
+      <c r="E6" t="inlineStr">
+        <is>
+          <t>DSI</t>
+        </is>
+      </c>
+      <c r="F6" t="inlineStr">
+        <is>
+          <t>28/08/2026</t>
+        </is>
+      </c>
+      <c r="G6" t="inlineStr">
+        <is>
+          <t>29/08/2026</t>
+        </is>
+      </c>
+      <c r="H6" t="inlineStr">
+        <is>
+          <t>Demandes</t>
+        </is>
+      </c>
+      <c r="I6" t="inlineStr">
+        <is>
+          <t>Compteur partagé, sans doublon</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>[Demandes] Rendre le coût présumé facultatif (100 %)</t>
+        </is>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>Livré</t>
+        </is>
+      </c>
+      <c r="C7" t="inlineStr">
+        <is>
+          <t>Terminé</t>
+        </is>
+      </c>
+      <c r="D7" t="inlineStr">
+        <is>
+          <t>Moyen</t>
+        </is>
+      </c>
+      <c r="E7" t="inlineStr">
+        <is>
+          <t>DSI</t>
+        </is>
+      </c>
+      <c r="F7" t="inlineStr">
+        <is>
+          <t>28/08/2026</t>
+        </is>
+      </c>
+      <c r="G7" t="inlineStr">
+        <is>
+          <t>01/09/2026</t>
+        </is>
+      </c>
+      <c r="H7" t="inlineStr">
+        <is>
+          <t>Demandes</t>
+        </is>
+      </c>
+      <c r="I7" t="inlineStr">
+        <is>
+          <t>Demande créable sans montant</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>[Fournisseurs] Catalogue fournisseurs (création, modification, statut) (100 %)</t>
+        </is>
+      </c>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>Livré</t>
+        </is>
+      </c>
+      <c r="C8" t="inlineStr">
+        <is>
+          <t>Terminé</t>
+        </is>
+      </c>
+      <c r="D8" t="inlineStr">
+        <is>
+          <t>Urgent</t>
+        </is>
+      </c>
+      <c r="E8" t="inlineStr">
+        <is>
+          <t>DSI</t>
+        </is>
+      </c>
+      <c r="F8" t="inlineStr">
+        <is>
+          <t>28/08/2026</t>
+        </is>
+      </c>
+      <c r="G8" t="inlineStr">
+        <is>
+          <t>30/08/2026</t>
+        </is>
+      </c>
+      <c r="H8" t="inlineStr">
+        <is>
+          <t>Fournisseurs</t>
+        </is>
+      </c>
+      <c r="I8" t="inlineStr">
+        <is>
+          <t>Nom, références, emplacement, WhatsApp, site</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>[Fournisseurs] Import des fournisseurs (Excel, CSV, JSON) (100 %)</t>
+        </is>
+      </c>
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>Livré</t>
+        </is>
+      </c>
+      <c r="C9" t="inlineStr">
+        <is>
+          <t>Terminé</t>
+        </is>
+      </c>
+      <c r="D9" t="inlineStr">
+        <is>
+          <t>Urgent</t>
+        </is>
+      </c>
+      <c r="E9" t="inlineStr">
+        <is>
+          <t>DSI</t>
+        </is>
+      </c>
+      <c r="F9" t="inlineStr">
+        <is>
+          <t>28/08/2026</t>
+        </is>
+      </c>
+      <c r="G9" t="inlineStr">
+        <is>
+          <t>30/08/2026</t>
+        </is>
+      </c>
+      <c r="H9" t="inlineStr">
+        <is>
+          <t>Fournisseurs</t>
+        </is>
+      </c>
+      <c r="I9" t="inlineStr">
+        <is>
+          <t>Aperçu, lignes invalides signalées</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>[Fournisseurs] Export des fournisseurs et modèles de fichiers (100 %)</t>
+        </is>
+      </c>
+      <c r="B10" t="inlineStr">
+        <is>
+          <t>Livré</t>
+        </is>
+      </c>
+      <c r="C10" t="inlineStr">
+        <is>
+          <t>Terminé</t>
+        </is>
+      </c>
+      <c r="D10" t="inlineStr">
+        <is>
+          <t>Moyen</t>
+        </is>
+      </c>
+      <c r="E10" t="inlineStr">
+        <is>
+          <t>DSI</t>
+        </is>
+      </c>
+      <c r="F10" t="inlineStr">
+        <is>
+          <t>28/08/2026</t>
+        </is>
+      </c>
+      <c r="G10" t="inlineStr">
+        <is>
+          <t>30/08/2026</t>
+        </is>
+      </c>
+      <c r="H10" t="inlineStr">
+        <is>
+          <t>Fournisseurs</t>
+        </is>
+      </c>
+      <c r="I10" t="inlineStr">
+        <is>
+          <t>Excel, JSON, CSV</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>[Négociation] Grille de négociation article × fournisseur (100 %)</t>
+        </is>
+      </c>
+      <c r="B11" t="inlineStr">
+        <is>
+          <t>Livré</t>
+        </is>
+      </c>
+      <c r="C11" t="inlineStr">
+        <is>
+          <t>Terminé</t>
+        </is>
+      </c>
+      <c r="D11" t="inlineStr">
+        <is>
+          <t>Urgent</t>
+        </is>
+      </c>
+      <c r="E11" t="inlineStr">
+        <is>
+          <t>DSI</t>
+        </is>
+      </c>
+      <c r="F11" t="inlineStr">
+        <is>
+          <t>28/08/2026</t>
+        </is>
+      </c>
+      <c r="G11" t="inlineStr">
+        <is>
+          <t>31/08/2026</t>
+        </is>
+      </c>
+      <c r="H11" t="inlineStr">
+        <is>
+          <t>Négociation</t>
+        </is>
+      </c>
+      <c r="I11" t="inlineStr">
+        <is>
+          <t>Un prix par article et par fournisseur</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="inlineStr">
+        <is>
+          <t>[Négociation] Rendre les prix facultatifs (seuil paramétrable) (100 %)</t>
+        </is>
+      </c>
+      <c r="B12" t="inlineStr">
+        <is>
+          <t>Livré</t>
+        </is>
+      </c>
+      <c r="C12" t="inlineStr">
+        <is>
+          <t>Terminé</t>
+        </is>
+      </c>
+      <c r="D12" t="inlineStr">
+        <is>
+          <t>Urgent</t>
+        </is>
+      </c>
+      <c r="E12" t="inlineStr">
+        <is>
+          <t>DSI</t>
+        </is>
+      </c>
+      <c r="F12" t="inlineStr">
+        <is>
+          <t>28/08/2026</t>
+        </is>
+      </c>
+      <c r="G12" t="inlineStr">
+        <is>
+          <t>02/09/2026</t>
+        </is>
+      </c>
+      <c r="H12" t="inlineStr">
+        <is>
+          <t>Négociation</t>
+        </is>
+      </c>
+      <c r="I12" t="inlineStr">
+        <is>
+          <t>Seuil 0 = facultatif</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="inlineStr">
+        <is>
+          <t>[Négociation] Coût total rendu (remise, TVA, frais de livraison) (100 %)</t>
+        </is>
+      </c>
+      <c r="B13" t="inlineStr">
+        <is>
+          <t>Livré</t>
+        </is>
+      </c>
+      <c r="C13" t="inlineStr">
+        <is>
+          <t>Terminé</t>
+        </is>
+      </c>
+      <c r="D13" t="inlineStr">
+        <is>
+          <t>Urgent</t>
+        </is>
+      </c>
+      <c r="E13" t="inlineStr">
+        <is>
+          <t>DSI</t>
+        </is>
+      </c>
+      <c r="F13" t="inlineStr">
+        <is>
+          <t>28/08/2026</t>
+        </is>
+      </c>
+      <c r="G13" t="inlineStr">
+        <is>
+          <t>31/08/2026</t>
+        </is>
+      </c>
+      <c r="H13" t="inlineStr">
+        <is>
+          <t>Négociation</t>
+        </is>
+      </c>
+      <c r="I13" t="inlineStr">
+        <is>
+          <t>Comparaison fiable des offres</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="inlineStr">
+        <is>
+          <t>[Comparaison] Score multicritère /100 et classement (100 %)</t>
+        </is>
+      </c>
+      <c r="B14" t="inlineStr">
+        <is>
+          <t>Livré</t>
+        </is>
+      </c>
+      <c r="C14" t="inlineStr">
+        <is>
+          <t>Terminé</t>
+        </is>
+      </c>
+      <c r="D14" t="inlineStr">
+        <is>
+          <t>Moyen</t>
+        </is>
+      </c>
+      <c r="E14" t="inlineStr">
+        <is>
+          <t>DSI</t>
+        </is>
+      </c>
+      <c r="F14" t="inlineStr">
+        <is>
+          <t>28/08/2026</t>
+        </is>
+      </c>
+      <c r="G14" t="inlineStr">
+        <is>
+          <t>31/08/2026</t>
+        </is>
+      </c>
+      <c r="H14" t="inlineStr">
+        <is>
+          <t>Négociation</t>
+        </is>
+      </c>
+      <c r="I14" t="inlineStr">
+        <is>
+          <t>Prix, délai, garantie, paiement</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="inlineStr">
+        <is>
+          <t>[Comparaison] Tableau croisé et meilleurs prix surlignés (100 %)</t>
+        </is>
+      </c>
+      <c r="B15" t="inlineStr">
+        <is>
+          <t>Livré</t>
+        </is>
+      </c>
+      <c r="C15" t="inlineStr">
+        <is>
+          <t>Terminé</t>
+        </is>
+      </c>
+      <c r="D15" t="inlineStr">
+        <is>
+          <t>Urgent</t>
+        </is>
+      </c>
+      <c r="E15" t="inlineStr">
+        <is>
+          <t>DSI</t>
+        </is>
+      </c>
+      <c r="F15" t="inlineStr">
+        <is>
+          <t>28/08/2026</t>
+        </is>
+      </c>
+      <c r="G15" t="inlineStr">
+        <is>
+          <t>31/08/2026</t>
+        </is>
+      </c>
+      <c r="H15" t="inlineStr">
+        <is>
+          <t>Négociation</t>
+        </is>
+      </c>
+      <c r="I15" t="inlineStr">
+        <is>
+          <t>Lecture seule, étape non bloquante</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="inlineStr">
+        <is>
+          <t>[Validation] Circuit de validation (approuver / refuser / modifier) (100 %)</t>
+        </is>
+      </c>
+      <c r="B16" t="inlineStr">
+        <is>
+          <t>Livré</t>
+        </is>
+      </c>
+      <c r="C16" t="inlineStr">
+        <is>
+          <t>Terminé</t>
+        </is>
+      </c>
+      <c r="D16" t="inlineStr">
+        <is>
+          <t>Urgent</t>
+        </is>
+      </c>
+      <c r="E16" t="inlineStr">
+        <is>
+          <t>DSI</t>
+        </is>
+      </c>
+      <c r="F16" t="inlineStr">
+        <is>
+          <t>28/08/2026</t>
+        </is>
+      </c>
+      <c r="G16" t="inlineStr">
+        <is>
+          <t>01/09/2026</t>
+        </is>
+      </c>
+      <c r="H16" t="inlineStr">
+        <is>
+          <t>Validation</t>
+        </is>
+      </c>
+      <c r="I16" t="inlineStr">
+        <is>
+          <t>Motif obligatoire si refus</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="inlineStr">
+        <is>
+          <t>[Commandes] Bons de commande BC-AAAA-NNNNN et confirmation (100 %)</t>
+        </is>
+      </c>
+      <c r="B17" t="inlineStr">
+        <is>
+          <t>Livré</t>
+        </is>
+      </c>
+      <c r="C17" t="inlineStr">
+        <is>
+          <t>Terminé</t>
+        </is>
+      </c>
+      <c r="D17" t="inlineStr">
+        <is>
+          <t>Urgent</t>
+        </is>
+      </c>
+      <c r="E17" t="inlineStr">
+        <is>
+          <t>DSI</t>
+        </is>
+      </c>
+      <c r="F17" t="inlineStr">
+        <is>
+          <t>28/08/2026</t>
+        </is>
+      </c>
+      <c r="G17" t="inlineStr">
+        <is>
+          <t>01/09/2026</t>
+        </is>
+      </c>
+      <c r="H17" t="inlineStr">
+        <is>
+          <t>Commandes</t>
+        </is>
+      </c>
+      <c r="I17" t="inlineStr">
+        <is>
+          <t>Lignes aux prix négociés</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" t="inlineStr">
+        <is>
+          <t>[Commandes] Commande et impression sans fournisseur ni prix (100 %)</t>
+        </is>
+      </c>
+      <c r="B18" t="inlineStr">
+        <is>
+          <t>Livré</t>
+        </is>
+      </c>
+      <c r="C18" t="inlineStr">
+        <is>
+          <t>Terminé</t>
+        </is>
+      </c>
+      <c r="D18" t="inlineStr">
+        <is>
+          <t>Moyen</t>
+        </is>
+      </c>
+      <c r="E18" t="inlineStr">
+        <is>
+          <t>DSI</t>
+        </is>
+      </c>
+      <c r="F18" t="inlineStr">
+        <is>
+          <t>28/08/2026</t>
+        </is>
+      </c>
+      <c r="G18" t="inlineStr">
+        <is>
+          <t>02/09/2026</t>
+        </is>
+      </c>
+      <c r="H18" t="inlineStr">
+        <is>
+          <t>Commandes</t>
+        </is>
+      </c>
+      <c r="I18" t="inlineStr">
+        <is>
+          <t>Cas des consultations en cours</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" t="inlineStr">
+        <is>
+          <t>[Réceptions] Réceptions complètes et partielles (100 %)</t>
+        </is>
+      </c>
+      <c r="B19" t="inlineStr">
+        <is>
+          <t>Livré</t>
+        </is>
+      </c>
+      <c r="C19" t="inlineStr">
+        <is>
+          <t>Terminé</t>
+        </is>
+      </c>
+      <c r="D19" t="inlineStr">
+        <is>
+          <t>Urgent</t>
+        </is>
+      </c>
+      <c r="E19" t="inlineStr">
+        <is>
+          <t>DSI</t>
+        </is>
+      </c>
+      <c r="F19" t="inlineStr">
+        <is>
+          <t>28/08/2026</t>
+        </is>
+      </c>
+      <c r="G19" t="inlineStr">
+        <is>
+          <t>01/09/2026</t>
+        </is>
+      </c>
+      <c r="H19" t="inlineStr">
+        <is>
+          <t>Commandes</t>
+        </is>
+      </c>
+      <c r="I19" t="inlineStr">
+        <is>
+          <t>Clôture automatique si complète</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" t="inlineStr">
+        <is>
+          <t>[Administration] Suppressions (demande, commande, réception, utilisateur) (100 %)</t>
+        </is>
+      </c>
+      <c r="B20" t="inlineStr">
+        <is>
+          <t>Livré</t>
+        </is>
+      </c>
+      <c r="C20" t="inlineStr">
+        <is>
+          <t>Terminé</t>
+        </is>
+      </c>
+      <c r="D20" t="inlineStr">
+        <is>
+          <t>Urgent</t>
+        </is>
+      </c>
+      <c r="E20" t="inlineStr">
+        <is>
+          <t>DSI</t>
+        </is>
+      </c>
+      <c r="F20" t="inlineStr">
+        <is>
+          <t>28/08/2026</t>
+        </is>
+      </c>
+      <c r="G20" t="inlineStr">
+        <is>
+          <t>01/09/2026</t>
+        </is>
+      </c>
+      <c r="H20" t="inlineStr">
+        <is>
+          <t>Administration</t>
+        </is>
+      </c>
+      <c r="I20" t="inlineStr">
+        <is>
+          <t>Cascades et garde-fous</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" t="inlineStr">
+        <is>
+          <t>[Alertes] Notifications et relances automatiques (100 %)</t>
+        </is>
+      </c>
+      <c r="B21" t="inlineStr">
+        <is>
+          <t>Livré</t>
+        </is>
+      </c>
+      <c r="C21" t="inlineStr">
+        <is>
+          <t>Terminé</t>
+        </is>
+      </c>
+      <c r="D21" t="inlineStr">
+        <is>
+          <t>Urgent</t>
+        </is>
+      </c>
+      <c r="E21" t="inlineStr">
+        <is>
+          <t>DSI</t>
+        </is>
+      </c>
+      <c r="F21" t="inlineStr">
+        <is>
+          <t>28/08/2026</t>
+        </is>
+      </c>
+      <c r="G21" t="inlineStr">
+        <is>
+          <t>02/09/2026</t>
+        </is>
+      </c>
+      <c r="H21" t="inlineStr">
+        <is>
+          <t>Alertes</t>
+        </is>
+      </c>
+      <c r="I21" t="inlineStr">
+        <is>
+          <t>Validation et réception, anti-doublon</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" t="inlineStr">
+        <is>
+          <t>[Alertes] Bandeau d'alertes et pastilles sur le tableau de bord (100 %)</t>
+        </is>
+      </c>
+      <c r="B22" t="inlineStr">
+        <is>
+          <t>Livré</t>
+        </is>
+      </c>
+      <c r="C22" t="inlineStr">
+        <is>
+          <t>Terminé</t>
+        </is>
+      </c>
+      <c r="D22" t="inlineStr">
+        <is>
+          <t>Moyen</t>
+        </is>
+      </c>
+      <c r="E22" t="inlineStr">
+        <is>
+          <t>DSI</t>
+        </is>
+      </c>
+      <c r="F22" t="inlineStr">
+        <is>
+          <t>28/08/2026</t>
+        </is>
+      </c>
+      <c r="G22" t="inlineStr">
+        <is>
+          <t>02/09/2026</t>
+        </is>
+      </c>
+      <c r="H22" t="inlineStr">
+        <is>
+          <t>Alertes</t>
+        </is>
+      </c>
+      <c r="I22" t="inlineStr">
+        <is>
+          <t>Vue immédiate des retards</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" t="inlineStr">
+        <is>
+          <t>[Alertes] Sons de notification (3 niveaux) et volume réglable (100 %)</t>
+        </is>
+      </c>
+      <c r="B23" t="inlineStr">
+        <is>
+          <t>Livré</t>
+        </is>
+      </c>
+      <c r="C23" t="inlineStr">
+        <is>
+          <t>Terminé</t>
+        </is>
+      </c>
+      <c r="D23" t="inlineStr">
+        <is>
+          <t>Moyen</t>
+        </is>
+      </c>
+      <c r="E23" t="inlineStr">
+        <is>
+          <t>DSI</t>
+        </is>
+      </c>
+      <c r="F23" t="inlineStr">
+        <is>
+          <t>28/08/2026</t>
+        </is>
+      </c>
+      <c r="G23" t="inlineStr">
+        <is>
+          <t>02/09/2026</t>
+        </is>
+      </c>
+      <c r="H23" t="inlineStr">
+        <is>
+          <t>Alertes</t>
+        </is>
+      </c>
+      <c r="I23" t="inlineStr">
+        <is>
+          <t>Avec son de secours si bloqué</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" t="inlineStr">
+        <is>
+          <t>[Alertes] Alarme répétée jusqu'à lecture du message (100 %)</t>
+        </is>
+      </c>
+      <c r="B24" t="inlineStr">
+        <is>
+          <t>Livré</t>
+        </is>
+      </c>
+      <c r="C24" t="inlineStr">
+        <is>
+          <t>Terminé</t>
+        </is>
+      </c>
+      <c r="D24" t="inlineStr">
+        <is>
+          <t>Moyen</t>
+        </is>
+      </c>
+      <c r="E24" t="inlineStr">
+        <is>
+          <t>DSI</t>
+        </is>
+      </c>
+      <c r="F24" t="inlineStr">
+        <is>
+          <t>28/08/2026</t>
+        </is>
+      </c>
+      <c r="G24" t="inlineStr">
+        <is>
+          <t>02/09/2026</t>
+        </is>
+      </c>
+      <c r="H24" t="inlineStr">
+        <is>
+          <t>Alertes</t>
+        </is>
+      </c>
+      <c r="I24" t="inlineStr">
+        <is>
+          <t>15 s, maximum 10 répétitions</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" t="inlineStr">
+        <is>
+          <t>[Alertes] Notifications du navigateur (bulles système) (100 %)</t>
+        </is>
+      </c>
+      <c r="B25" t="inlineStr">
+        <is>
+          <t>Livré</t>
+        </is>
+      </c>
+      <c r="C25" t="inlineStr">
+        <is>
+          <t>Terminé</t>
+        </is>
+      </c>
+      <c r="D25" t="inlineStr">
+        <is>
+          <t>Moyen</t>
+        </is>
+      </c>
+      <c r="E25" t="inlineStr">
+        <is>
+          <t>DSI</t>
+        </is>
+      </c>
+      <c r="F25" t="inlineStr">
+        <is>
+          <t>28/08/2026</t>
+        </is>
+      </c>
+      <c r="G25" t="inlineStr">
+        <is>
+          <t>02/09/2026</t>
+        </is>
+      </c>
+      <c r="H25" t="inlineStr">
+        <is>
+          <t>Alertes</t>
+        </is>
+      </c>
+      <c r="I25" t="inlineStr">
+        <is>
+          <t>Actives onglet en arrière-plan</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" t="inlineStr">
+        <is>
+          <t>[Alertes] Alerte visuelle (onglet clignotant, pastille pulsante) (100 %)</t>
+        </is>
+      </c>
+      <c r="B26" t="inlineStr">
+        <is>
+          <t>Livré</t>
+        </is>
+      </c>
+      <c r="C26" t="inlineStr">
+        <is>
+          <t>Terminé</t>
+        </is>
+      </c>
+      <c r="D26" t="inlineStr">
+        <is>
+          <t>Moyen</t>
+        </is>
+      </c>
+      <c r="E26" t="inlineStr">
+        <is>
+          <t>DSI</t>
+        </is>
+      </c>
+      <c r="F26" t="inlineStr">
+        <is>
+          <t>28/08/2026</t>
+        </is>
+      </c>
+      <c r="G26" t="inlineStr">
+        <is>
+          <t>02/09/2026</t>
+        </is>
+      </c>
+      <c r="H26" t="inlineStr">
+        <is>
+          <t>Alertes</t>
+        </is>
+      </c>
+      <c r="I26" t="inlineStr">
+        <is>
+          <t>Secours si le son est coupé</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" t="inlineStr">
+        <is>
+          <t>[Documents] Impression fiche de demande et bon de commande (100 %)</t>
+        </is>
+      </c>
+      <c r="B27" t="inlineStr">
+        <is>
+          <t>Livré</t>
+        </is>
+      </c>
+      <c r="C27" t="inlineStr">
+        <is>
+          <t>Terminé</t>
+        </is>
+      </c>
+      <c r="D27" t="inlineStr">
+        <is>
+          <t>Urgent</t>
+        </is>
+      </c>
+      <c r="E27" t="inlineStr">
+        <is>
+          <t>DSI</t>
+        </is>
+      </c>
+      <c r="F27" t="inlineStr">
+        <is>
+          <t>28/08/2026</t>
+        </is>
+      </c>
+      <c r="G27" t="inlineStr">
+        <is>
+          <t>02/09/2026</t>
+        </is>
+      </c>
+      <c r="H27" t="inlineStr">
+        <is>
+          <t>Documents</t>
+        </is>
+      </c>
+      <c r="I27" t="inlineStr">
+        <is>
+          <t>Colonnes de prix vides à compléter</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" t="inlineStr">
+        <is>
+          <t>[Documents] Exports PDF (demandes, commandes, réceptions) (100 %)</t>
+        </is>
+      </c>
+      <c r="B28" t="inlineStr">
+        <is>
+          <t>Livré</t>
+        </is>
+      </c>
+      <c r="C28" t="inlineStr">
+        <is>
+          <t>Terminé</t>
+        </is>
+      </c>
+      <c r="D28" t="inlineStr">
+        <is>
+          <t>Urgent</t>
+        </is>
+      </c>
+      <c r="E28" t="inlineStr">
+        <is>
+          <t>DSI</t>
+        </is>
+      </c>
+      <c r="F28" t="inlineStr">
+        <is>
+          <t>28/08/2026</t>
+        </is>
+      </c>
+      <c r="G28" t="inlineStr">
+        <is>
+          <t>01/09/2026</t>
+        </is>
+      </c>
+      <c r="H28" t="inlineStr">
+        <is>
+          <t>Documents</t>
+        </is>
+      </c>
+      <c r="I28" t="inlineStr">
+        <is>
+          <t>jsPDF, repli impression</t>
+        </is>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" t="inlineStr">
+        <is>
+          <t>[Documents] Exports Excel et CSV (100 %)</t>
+        </is>
+      </c>
+      <c r="B29" t="inlineStr">
+        <is>
+          <t>Livré</t>
+        </is>
+      </c>
+      <c r="C29" t="inlineStr">
+        <is>
+          <t>Terminé</t>
+        </is>
+      </c>
+      <c r="D29" t="inlineStr">
+        <is>
+          <t>Moyen</t>
+        </is>
+      </c>
+      <c r="E29" t="inlineStr">
+        <is>
+          <t>DSI</t>
+        </is>
+      </c>
+      <c r="F29" t="inlineStr">
+        <is>
+          <t>28/08/2026</t>
+        </is>
+      </c>
+      <c r="G29" t="inlineStr">
+        <is>
+          <t>01/09/2026</t>
+        </is>
+      </c>
+      <c r="H29" t="inlineStr">
+        <is>
+          <t>Documents</t>
+        </is>
+      </c>
+      <c r="I29" t="inlineStr">
+        <is>
+          <t>Comparaison incluse</t>
+        </is>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" t="inlineStr">
+        <is>
+          <t>[Identité] Intégration du logo et charte violet / bleu nuit (100 %)</t>
+        </is>
+      </c>
+      <c r="B30" t="inlineStr">
+        <is>
+          <t>Livré</t>
+        </is>
+      </c>
+      <c r="C30" t="inlineStr">
+        <is>
+          <t>Terminé</t>
+        </is>
+      </c>
+      <c r="D30" t="inlineStr">
+        <is>
+          <t>Moyen</t>
+        </is>
+      </c>
+      <c r="E30" t="inlineStr">
+        <is>
+          <t>Direction</t>
+        </is>
+      </c>
+      <c r="F30" t="inlineStr">
+        <is>
+          <t>28/08/2026</t>
+        </is>
+      </c>
+      <c r="G30" t="inlineStr">
+        <is>
+          <t>02/09/2026</t>
+        </is>
+      </c>
+      <c r="H30" t="inlineStr">
+        <is>
+          <t>Documents</t>
+        </is>
+      </c>
+      <c r="I30" t="inlineStr">
+        <is>
+          <t>Site, impressions, PDF, favicon</t>
+        </is>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" t="inlineStr">
+        <is>
+          <t>[Données] Synchronisation Supabase en temps réel (100 %)</t>
+        </is>
+      </c>
+      <c r="B31" t="inlineStr">
+        <is>
+          <t>Livré</t>
+        </is>
+      </c>
+      <c r="C31" t="inlineStr">
+        <is>
+          <t>Terminé</t>
+        </is>
+      </c>
+      <c r="D31" t="inlineStr">
+        <is>
+          <t>Urgent</t>
+        </is>
+      </c>
+      <c r="E31" t="inlineStr">
+        <is>
+          <t>DSI</t>
+        </is>
+      </c>
+      <c r="F31" t="inlineStr">
+        <is>
+          <t>28/08/2026</t>
+        </is>
+      </c>
+      <c r="G31" t="inlineStr">
+        <is>
+          <t>02/09/2026</t>
+        </is>
+      </c>
+      <c r="H31" t="inlineStr">
+        <is>
+          <t>Données</t>
+        </is>
+      </c>
+      <c r="I31" t="inlineStr">
+        <is>
+          <t>Partage entre tous les postes</t>
+        </is>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" t="inlineStr">
+        <is>
+          <t>[Données] Sécurisation anti-écrasement entre appareils (100 %)</t>
+        </is>
+      </c>
+      <c r="B32" t="inlineStr">
+        <is>
+          <t>Livré</t>
+        </is>
+      </c>
+      <c r="C32" t="inlineStr">
+        <is>
+          <t>Terminé</t>
+        </is>
+      </c>
+      <c r="D32" t="inlineStr">
+        <is>
+          <t>Urgent</t>
+        </is>
+      </c>
+      <c r="E32" t="inlineStr">
+        <is>
+          <t>DSI</t>
+        </is>
+      </c>
+      <c r="F32" t="inlineStr">
+        <is>
+          <t>28/08/2026</t>
+        </is>
+      </c>
+      <c r="G32" t="inlineStr">
+        <is>
+          <t>02/09/2026</t>
+        </is>
+      </c>
+      <c r="H32" t="inlineStr">
+        <is>
+          <t>Données</t>
+        </is>
+      </c>
+      <c r="I32" t="inlineStr">
+        <is>
+          <t>Le serveur fait foi au démarrage</t>
+        </is>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" t="inlineStr">
+        <is>
+          <t>[Pilotage] Tableau de bord graphique (3 graphiques) (100 %)</t>
+        </is>
+      </c>
+      <c r="B33" t="inlineStr">
+        <is>
+          <t>Livré</t>
+        </is>
+      </c>
+      <c r="C33" t="inlineStr">
+        <is>
+          <t>Terminé</t>
+        </is>
+      </c>
+      <c r="D33" t="inlineStr">
+        <is>
+          <t>Moyen</t>
+        </is>
+      </c>
+      <c r="E33" t="inlineStr">
+        <is>
+          <t>DSI</t>
+        </is>
+      </c>
+      <c r="F33" t="inlineStr">
+        <is>
+          <t>28/08/2026</t>
+        </is>
+      </c>
+      <c r="G33" t="inlineStr">
+        <is>
+          <t>02/09/2026</t>
+        </is>
+      </c>
+      <c r="H33" t="inlineStr">
+        <is>
+          <t>Pilotage</t>
+        </is>
+      </c>
+      <c r="I33" t="inlineStr">
+        <is>
+          <t>Achats 12 mois, répartition, top 5</t>
+        </is>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" t="inlineStr">
+        <is>
+          <t>[Qualité] Suite de tests automatisés (197 contrôles) (100 %)</t>
+        </is>
+      </c>
+      <c r="B34" t="inlineStr">
+        <is>
+          <t>Livré</t>
+        </is>
+      </c>
+      <c r="C34" t="inlineStr">
+        <is>
+          <t>Terminé</t>
+        </is>
+      </c>
+      <c r="D34" t="inlineStr">
+        <is>
+          <t>Urgent</t>
+        </is>
+      </c>
+      <c r="E34" t="inlineStr">
+        <is>
+          <t>DSI</t>
+        </is>
+      </c>
+      <c r="F34" t="inlineStr">
+        <is>
+          <t>28/08/2026</t>
+        </is>
+      </c>
+      <c r="G34" t="inlineStr">
+        <is>
+          <t>02/09/2026</t>
+        </is>
+      </c>
+      <c r="H34" t="inlineStr">
+        <is>
+          <t>Qualité</t>
+        </is>
+      </c>
+      <c r="I34" t="inlineStr">
+        <is>
+          <t>13 séries, exécutées avant publication</t>
+        </is>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" t="inlineStr">
+        <is>
+          <t>[Déploiement] Déploiement continu GitHub vers Vercel (100 %)</t>
+        </is>
+      </c>
+      <c r="B35" t="inlineStr">
+        <is>
+          <t>Livré</t>
+        </is>
+      </c>
+      <c r="C35" t="inlineStr">
+        <is>
+          <t>Terminé</t>
+        </is>
+      </c>
+      <c r="D35" t="inlineStr">
+        <is>
+          <t>Urgent</t>
+        </is>
+      </c>
+      <c r="E35" t="inlineStr">
+        <is>
+          <t>DSI</t>
+        </is>
+      </c>
+      <c r="F35" t="inlineStr">
+        <is>
+          <t>28/08/2026</t>
+        </is>
+      </c>
+      <c r="G35" t="inlineStr">
+        <is>
+          <t>02/09/2026</t>
+        </is>
+      </c>
+      <c r="H35" t="inlineStr">
+        <is>
+          <t>Déploiement</t>
+        </is>
+      </c>
+      <c r="I35" t="inlineStr">
+        <is>
+          <t>Une commande : scripts/publish.mjs</t>
+        </is>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" t="inlineStr">
+        <is>
+          <t>[Documentation] Cahier des charges et synthèse direction (100 %)</t>
+        </is>
+      </c>
+      <c r="B36" t="inlineStr">
+        <is>
+          <t>Livré</t>
+        </is>
+      </c>
+      <c r="C36" t="inlineStr">
+        <is>
+          <t>Terminé</t>
+        </is>
+      </c>
+      <c r="D36" t="inlineStr">
+        <is>
+          <t>Moyen</t>
+        </is>
+      </c>
+      <c r="E36" t="inlineStr">
+        <is>
+          <t>DSI</t>
+        </is>
+      </c>
+      <c r="F36" t="inlineStr">
+        <is>
+          <t>28/08/2026</t>
+        </is>
+      </c>
+      <c r="G36" t="inlineStr">
+        <is>
+          <t>02/09/2026</t>
+        </is>
+      </c>
+      <c r="H36" t="inlineStr">
+        <is>
+          <t>Documentation</t>
+        </is>
+      </c>
+      <c r="I36" t="inlineStr">
+        <is>
+          <t>PDF et Word, 14 et 4 pages</t>
+        </is>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" t="inlineStr">
+        <is>
+          <t>[Qualité] Recette utilisateur et ajustements (60 %)</t>
+        </is>
+      </c>
+      <c r="B37" t="inlineStr">
+        <is>
+          <t>En cours</t>
+        </is>
+      </c>
+      <c r="C37" t="inlineStr">
+        <is>
+          <t>En cours</t>
+        </is>
+      </c>
+      <c r="D37" t="inlineStr">
+        <is>
+          <t>Urgent</t>
+        </is>
+      </c>
+      <c r="E37" t="inlineStr">
+        <is>
+          <t>Direction</t>
+        </is>
+      </c>
+      <c r="F37" t="inlineStr">
+        <is>
+          <t>28/08/2026</t>
+        </is>
+      </c>
+      <c r="G37" t="inlineStr">
+        <is>
+          <t>05/09/2026</t>
+        </is>
+      </c>
+      <c r="H37" t="inlineStr">
+        <is>
+          <t>Qualité</t>
+        </is>
+      </c>
+      <c r="I37" t="inlineStr">
+        <is>
+          <t>Retours des utilisateurs finaux</t>
+        </is>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" t="inlineStr">
+        <is>
+          <t>[Sécurité] Durcissement des politiques d'accès (RLS) (30 %)</t>
+        </is>
+      </c>
+      <c r="B38" t="inlineStr">
+        <is>
+          <t>En cours</t>
+        </is>
+      </c>
+      <c r="C38" t="inlineStr">
+        <is>
+          <t>En cours</t>
+        </is>
+      </c>
+      <c r="D38" t="inlineStr">
+        <is>
+          <t>Urgent</t>
+        </is>
+      </c>
+      <c r="E38" t="inlineStr">
+        <is>
+          <t>DSI</t>
+        </is>
+      </c>
+      <c r="F38" t="inlineStr">
+        <is>
+          <t>28/08/2026</t>
+        </is>
+      </c>
+      <c r="G38" t="inlineStr">
+        <is>
+          <t>09/09/2026</t>
+        </is>
+      </c>
+      <c r="H38" t="inlineStr">
+        <is>
+          <t>Sécurité</t>
+        </is>
+      </c>
+      <c r="I38" t="inlineStr">
+        <is>
+          <t>Restreindre par rôle avant généralisation</t>
+        </is>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" t="inlineStr">
+        <is>
+          <t>[Sécurité] Journal d'audit des actions sensibles (15 %)</t>
+        </is>
+      </c>
+      <c r="B39" t="inlineStr">
+        <is>
+          <t>En cours</t>
+        </is>
+      </c>
+      <c r="C39" t="inlineStr">
+        <is>
+          <t>En cours</t>
+        </is>
+      </c>
+      <c r="D39" t="inlineStr">
+        <is>
+          <t>Urgent</t>
+        </is>
+      </c>
+      <c r="E39" t="inlineStr">
+        <is>
+          <t>DSI</t>
+        </is>
+      </c>
+      <c r="F39" t="inlineStr">
+        <is>
+          <t>28/08/2026</t>
+        </is>
+      </c>
+      <c r="G39" t="inlineStr">
+        <is>
+          <t>12/09/2026</t>
+        </is>
+      </c>
+      <c r="H39" t="inlineStr">
+        <is>
+          <t>Sécurité</t>
+        </is>
+      </c>
+      <c r="I39" t="inlineStr">
+        <is>
+          <t>Qui a supprimé/modifié quoi et quand</t>
+        </is>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" t="inlineStr">
+        <is>
+          <t>[Sécurité] Authentification sécurisée (mots de passe hachés) (0 %)</t>
+        </is>
+      </c>
+      <c r="B40" t="inlineStr">
+        <is>
+          <t>Planifié</t>
+        </is>
+      </c>
+      <c r="C40" t="inlineStr">
+        <is>
+          <t>Pas commencé</t>
+        </is>
+      </c>
+      <c r="D40" t="inlineStr">
+        <is>
+          <t>Urgent</t>
+        </is>
+      </c>
+      <c r="E40" t="inlineStr">
+        <is>
+          <t>DSI</t>
+        </is>
+      </c>
+      <c r="F40" t="inlineStr"/>
+      <c r="G40" t="inlineStr">
+        <is>
+          <t>19/09/2026</t>
+        </is>
+      </c>
+      <c r="H40" t="inlineStr">
+        <is>
+          <t>Sécurité</t>
+        </is>
+      </c>
+      <c r="I40" t="inlineStr">
+        <is>
+          <t>Migration vers Supabase Auth</t>
+        </is>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" t="inlineStr">
+        <is>
+          <t>[Alertes] Notifications par e-mail (0 %)</t>
+        </is>
+      </c>
+      <c r="B41" t="inlineStr">
+        <is>
+          <t>Planifié</t>
+        </is>
+      </c>
+      <c r="C41" t="inlineStr">
+        <is>
+          <t>Pas commencé</t>
+        </is>
+      </c>
+      <c r="D41" t="inlineStr">
+        <is>
+          <t>Moyen</t>
+        </is>
+      </c>
+      <c r="E41" t="inlineStr">
+        <is>
+          <t>DSI</t>
+        </is>
+      </c>
+      <c r="F41" t="inlineStr"/>
+      <c r="G41" t="inlineStr">
+        <is>
+          <t>26/09/2026</t>
+        </is>
+      </c>
+      <c r="H41" t="inlineStr">
+        <is>
+          <t>Alertes</t>
+        </is>
+      </c>
+      <c r="I41" t="inlineStr">
+        <is>
+          <t>Réduction des délais de réponse</t>
+        </is>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" t="inlineStr">
+        <is>
+          <t>[Pilotage] Budgets par service avec alerte de dépassement (0 %)</t>
+        </is>
+      </c>
+      <c r="B42" t="inlineStr">
+        <is>
+          <t>Planifié</t>
+        </is>
+      </c>
+      <c r="C42" t="inlineStr">
+        <is>
+          <t>Pas commencé</t>
+        </is>
+      </c>
+      <c r="D42" t="inlineStr">
+        <is>
+          <t>Moyen</t>
+        </is>
+      </c>
+      <c r="E42" t="inlineStr">
+        <is>
+          <t>Direction</t>
+        </is>
+      </c>
+      <c r="F42" t="inlineStr"/>
+      <c r="G42" t="inlineStr">
+        <is>
+          <t>10/10/2026</t>
+        </is>
+      </c>
+      <c r="H42" t="inlineStr">
+        <is>
+          <t>Pilotage</t>
+        </is>
+      </c>
+      <c r="I42" t="inlineStr">
+        <is>
+          <t>Pilotage financier</t>
+        </is>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43" t="inlineStr">
+        <is>
+          <t>[Fournisseurs] Portail fournisseur (saisie directe des offres) (0 %)</t>
+        </is>
+      </c>
+      <c r="B43" t="inlineStr">
+        <is>
+          <t>Planifié</t>
+        </is>
+      </c>
+      <c r="C43" t="inlineStr">
+        <is>
+          <t>Pas commencé</t>
+        </is>
+      </c>
+      <c r="D43" t="inlineStr">
+        <is>
+          <t>Faible</t>
+        </is>
+      </c>
+      <c r="E43" t="inlineStr">
+        <is>
+          <t>DSI</t>
+        </is>
+      </c>
+      <c r="F43" t="inlineStr"/>
+      <c r="G43" t="inlineStr">
+        <is>
+          <t>24/10/2026</t>
+        </is>
+      </c>
+      <c r="H43" t="inlineStr">
+        <is>
+          <t>Fournisseurs</t>
+        </is>
+      </c>
+      <c r="I43" t="inlineStr">
+        <is>
+          <t>Productivité sur les consultations</t>
+        </is>
+      </c>
+    </row>
+    <row r="44">
+      <c r="A44" t="inlineStr">
+        <is>
+          <t>[Logistique] Gestion des stocks liée aux réceptions (0 %)</t>
+        </is>
+      </c>
+      <c r="B44" t="inlineStr">
+        <is>
+          <t>Planifié</t>
+        </is>
+      </c>
+      <c r="C44" t="inlineStr">
+        <is>
+          <t>Pas commencé</t>
+        </is>
+      </c>
+      <c r="D44" t="inlineStr">
+        <is>
+          <t>Faible</t>
+        </is>
+      </c>
+      <c r="E44" t="inlineStr">
+        <is>
+          <t>Logistique</t>
+        </is>
+      </c>
+      <c r="F44" t="inlineStr"/>
+      <c r="G44" t="inlineStr">
+        <is>
+          <t>31/10/2026</t>
+        </is>
+      </c>
+      <c r="H44" t="inlineStr">
+        <is>
+          <t>Pilotage</t>
+        </is>
+      </c>
+      <c r="I44" t="inlineStr">
+        <is>
+          <t>À cadrer</t>
+        </is>
+      </c>
+    </row>
+    <row r="45">
+      <c r="A45" t="inlineStr">
+        <is>
+          <t>[Sécurité] Authentification unique (SSO) (0 %)</t>
+        </is>
+      </c>
+      <c r="B45" t="inlineStr">
+        <is>
+          <t>Planifié</t>
+        </is>
+      </c>
+      <c r="C45" t="inlineStr">
+        <is>
+          <t>Pas commencé</t>
+        </is>
+      </c>
+      <c r="D45" t="inlineStr">
+        <is>
+          <t>Faible</t>
+        </is>
+      </c>
+      <c r="E45" t="inlineStr">
+        <is>
+          <t>DSI</t>
+        </is>
+      </c>
+      <c r="F45" t="inlineStr"/>
+      <c r="G45" t="inlineStr">
+        <is>
+          <t>31/10/2026</t>
+        </is>
+      </c>
+      <c r="H45" t="inlineStr">
+        <is>
+          <t>Sécurité</t>
+        </is>
+      </c>
+      <c r="I45" t="inlineStr">
+        <is>
+          <t>Confort utilisateur</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+  <tableParts count="1">
+    <tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>
+  </tableParts>
+</worksheet>
 </file>
</xml_diff>

<commit_message>
Planner : colonnes Developpement / Test / Pilote / Deploiement + taches par etape et checklists
</commit_message>
<xml_diff>
--- a/docs/planner/VOOMNET-planner.xlsx
+++ b/docs/planner/VOOMNET-planner.xlsx
@@ -209,18 +209,22 @@
 </file>
 
 <file path=xl/tables/table2.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="2" name="GrilleVOOMNET" displayName="GrilleVOOMNET" ref="A1:I45" headerRowCount="1">
-  <autoFilter ref="A1:I45"/>
-  <tableColumns count="9">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="2" name="GrilleVOOMNET" displayName="GrilleVOOMNET" ref="A1:M45" headerRowCount="1">
+  <autoFilter ref="A1:M45"/>
+  <tableColumns count="13">
     <tableColumn id="1" name="Nom de la tâche"/>
     <tableColumn id="2" name="Compartiment"/>
     <tableColumn id="3" name="Progression"/>
-    <tableColumn id="4" name="Priorité"/>
-    <tableColumn id="5" name="Assigné à"/>
-    <tableColumn id="6" name="Date de début"/>
-    <tableColumn id="7" name="Date d'échéance"/>
-    <tableColumn id="8" name="Étiquettes"/>
-    <tableColumn id="9" name="Description"/>
+    <tableColumn id="4" name="Développement"/>
+    <tableColumn id="5" name="Test"/>
+    <tableColumn id="6" name="Pilote"/>
+    <tableColumn id="7" name="Déploiement"/>
+    <tableColumn id="8" name="Priorité"/>
+    <tableColumn id="9" name="Assigné à"/>
+    <tableColumn id="10" name="Date de début"/>
+    <tableColumn id="11" name="Date d'échéance"/>
+    <tableColumn id="12" name="Étiquettes"/>
+    <tableColumn id="13" name="Description"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium12" showRowStripes="1"/>
 </table>
@@ -5010,18 +5014,22 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I45"/>
+  <dimension ref="A1:M45"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="58" customWidth="1" min="1" max="1"/>
     <col width="15" customWidth="1" min="2" max="2"/>
     <col width="14" customWidth="1" min="3" max="3"/>
-    <col width="11" customWidth="1" min="4" max="4"/>
-    <col width="14" customWidth="1" min="5" max="5"/>
-    <col width="13" customWidth="1" min="6" max="6"/>
-    <col width="14" customWidth="1" min="7" max="7"/>
-    <col width="16" customWidth="1" min="8" max="8"/>
-    <col width="46" customWidth="1" min="9" max="9"/>
+    <col width="15" customWidth="1" min="4" max="4"/>
+    <col width="10" customWidth="1" min="5" max="5"/>
+    <col width="10" customWidth="1" min="6" max="6"/>
+    <col width="16" customWidth="1" min="7" max="7"/>
+    <col width="11" customWidth="1" min="8" max="8"/>
+    <col width="14" customWidth="1" min="9" max="9"/>
+    <col width="13" customWidth="1" min="10" max="10"/>
+    <col width="14" customWidth="1" min="11" max="11"/>
+    <col width="16" customWidth="1" min="12" max="12"/>
+    <col width="46" customWidth="1" min="13" max="13"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -5042,30 +5050,50 @@
       </c>
       <c r="D1" s="12" t="inlineStr">
         <is>
+          <t>Développement</t>
+        </is>
+      </c>
+      <c r="E1" s="12" t="inlineStr">
+        <is>
+          <t>Test</t>
+        </is>
+      </c>
+      <c r="F1" s="12" t="inlineStr">
+        <is>
+          <t>Pilote</t>
+        </is>
+      </c>
+      <c r="G1" s="12" t="inlineStr">
+        <is>
+          <t>Déploiement</t>
+        </is>
+      </c>
+      <c r="H1" s="12" t="inlineStr">
+        <is>
           <t>Priorité</t>
         </is>
       </c>
-      <c r="E1" s="12" t="inlineStr">
+      <c r="I1" s="12" t="inlineStr">
         <is>
           <t>Assigné à</t>
         </is>
       </c>
-      <c r="F1" s="12" t="inlineStr">
+      <c r="J1" s="12" t="inlineStr">
         <is>
           <t>Date de début</t>
         </is>
       </c>
-      <c r="G1" s="12" t="inlineStr">
+      <c r="K1" s="12" t="inlineStr">
         <is>
           <t>Date d'échéance</t>
         </is>
       </c>
-      <c r="H1" s="12" t="inlineStr">
+      <c r="L1" s="12" t="inlineStr">
         <is>
           <t>Étiquettes</t>
         </is>
       </c>
-      <c r="I1" s="12" t="inlineStr">
+      <c r="M1" s="12" t="inlineStr">
         <is>
           <t>Description</t>
         </is>
@@ -5089,30 +5117,50 @@
       </c>
       <c r="D2" t="inlineStr">
         <is>
+          <t>Terminé</t>
+        </is>
+      </c>
+      <c r="E2" t="inlineStr">
+        <is>
+          <t>Terminé</t>
+        </is>
+      </c>
+      <c r="F2" t="inlineStr">
+        <is>
+          <t>Terminé</t>
+        </is>
+      </c>
+      <c r="G2" t="inlineStr">
+        <is>
+          <t>Terminé</t>
+        </is>
+      </c>
+      <c r="H2" t="inlineStr">
+        <is>
           <t>Urgent</t>
         </is>
       </c>
-      <c r="E2" t="inlineStr">
+      <c r="I2" t="inlineStr">
         <is>
           <t>Projet</t>
         </is>
       </c>
-      <c r="F2" t="inlineStr">
+      <c r="J2" t="inlineStr">
         <is>
           <t>28/08/2026</t>
         </is>
       </c>
-      <c r="G2" t="inlineStr">
+      <c r="K2" t="inlineStr">
         <is>
           <t>28/08/2026</t>
         </is>
       </c>
-      <c r="H2" t="inlineStr">
+      <c r="L2" t="inlineStr">
         <is>
           <t>Cadrage</t>
         </is>
       </c>
-      <c r="I2" t="inlineStr">
+      <c r="M2" t="inlineStr">
         <is>
           <t>Objectifs, périmètre, règles de gestion</t>
         </is>
@@ -5136,30 +5184,50 @@
       </c>
       <c r="D3" t="inlineStr">
         <is>
+          <t>Terminé</t>
+        </is>
+      </c>
+      <c r="E3" t="inlineStr">
+        <is>
+          <t>Terminé</t>
+        </is>
+      </c>
+      <c r="F3" t="inlineStr">
+        <is>
+          <t>Terminé</t>
+        </is>
+      </c>
+      <c r="G3" t="inlineStr">
+        <is>
+          <t>Terminé</t>
+        </is>
+      </c>
+      <c r="H3" t="inlineStr">
+        <is>
           <t>Urgent</t>
         </is>
       </c>
-      <c r="E3" t="inlineStr">
-        <is>
-          <t>DSI</t>
-        </is>
-      </c>
-      <c r="F3" t="inlineStr">
+      <c r="I3" t="inlineStr">
+        <is>
+          <t>DSI</t>
+        </is>
+      </c>
+      <c r="J3" t="inlineStr">
         <is>
           <t>28/08/2026</t>
         </is>
       </c>
-      <c r="G3" t="inlineStr">
+      <c r="K3" t="inlineStr">
         <is>
           <t>28/08/2026</t>
         </is>
       </c>
-      <c r="H3" t="inlineStr">
+      <c r="L3" t="inlineStr">
         <is>
           <t>Cadrage</t>
         </is>
       </c>
-      <c r="I3" t="inlineStr">
+      <c r="M3" t="inlineStr">
         <is>
           <t>Application web + base temps réel</t>
         </is>
@@ -5183,30 +5251,50 @@
       </c>
       <c r="D4" t="inlineStr">
         <is>
+          <t>Terminé</t>
+        </is>
+      </c>
+      <c r="E4" t="inlineStr">
+        <is>
+          <t>Terminé</t>
+        </is>
+      </c>
+      <c r="F4" t="inlineStr">
+        <is>
+          <t>Terminé</t>
+        </is>
+      </c>
+      <c r="G4" t="inlineStr">
+        <is>
+          <t>Terminé</t>
+        </is>
+      </c>
+      <c r="H4" t="inlineStr">
+        <is>
           <t>Urgent</t>
         </is>
       </c>
-      <c r="E4" t="inlineStr">
-        <is>
-          <t>DSI</t>
-        </is>
-      </c>
-      <c r="F4" t="inlineStr">
+      <c r="I4" t="inlineStr">
+        <is>
+          <t>DSI</t>
+        </is>
+      </c>
+      <c r="J4" t="inlineStr">
         <is>
           <t>28/08/2026</t>
         </is>
       </c>
-      <c r="G4" t="inlineStr">
+      <c r="K4" t="inlineStr">
         <is>
           <t>29/08/2026</t>
         </is>
       </c>
-      <c r="H4" t="inlineStr">
+      <c r="L4" t="inlineStr">
         <is>
           <t>Sécurité</t>
         </is>
       </c>
-      <c r="I4" t="inlineStr">
+      <c r="M4" t="inlineStr">
         <is>
           <t>Demandeur / Responsable / Administrateur</t>
         </is>
@@ -5230,30 +5318,50 @@
       </c>
       <c r="D5" t="inlineStr">
         <is>
+          <t>Terminé</t>
+        </is>
+      </c>
+      <c r="E5" t="inlineStr">
+        <is>
+          <t>Terminé</t>
+        </is>
+      </c>
+      <c r="F5" t="inlineStr">
+        <is>
+          <t>Terminé</t>
+        </is>
+      </c>
+      <c r="G5" t="inlineStr">
+        <is>
+          <t>Terminé</t>
+        </is>
+      </c>
+      <c r="H5" t="inlineStr">
+        <is>
           <t>Urgent</t>
         </is>
       </c>
-      <c r="E5" t="inlineStr">
-        <is>
-          <t>DSI</t>
-        </is>
-      </c>
-      <c r="F5" t="inlineStr">
+      <c r="I5" t="inlineStr">
+        <is>
+          <t>DSI</t>
+        </is>
+      </c>
+      <c r="J5" t="inlineStr">
         <is>
           <t>28/08/2026</t>
         </is>
       </c>
-      <c r="G5" t="inlineStr">
+      <c r="K5" t="inlineStr">
         <is>
           <t>29/08/2026</t>
         </is>
       </c>
-      <c r="H5" t="inlineStr">
+      <c r="L5" t="inlineStr">
         <is>
           <t>Demandes</t>
         </is>
       </c>
-      <c r="I5" t="inlineStr">
+      <c r="M5" t="inlineStr">
         <is>
           <t>Création, brouillon, reprise</t>
         </is>
@@ -5277,30 +5385,50 @@
       </c>
       <c r="D6" t="inlineStr">
         <is>
+          <t>Terminé</t>
+        </is>
+      </c>
+      <c r="E6" t="inlineStr">
+        <is>
+          <t>Terminé</t>
+        </is>
+      </c>
+      <c r="F6" t="inlineStr">
+        <is>
+          <t>Terminé</t>
+        </is>
+      </c>
+      <c r="G6" t="inlineStr">
+        <is>
+          <t>Terminé</t>
+        </is>
+      </c>
+      <c r="H6" t="inlineStr">
+        <is>
           <t>Urgent</t>
         </is>
       </c>
-      <c r="E6" t="inlineStr">
-        <is>
-          <t>DSI</t>
-        </is>
-      </c>
-      <c r="F6" t="inlineStr">
+      <c r="I6" t="inlineStr">
+        <is>
+          <t>DSI</t>
+        </is>
+      </c>
+      <c r="J6" t="inlineStr">
         <is>
           <t>28/08/2026</t>
         </is>
       </c>
-      <c r="G6" t="inlineStr">
+      <c r="K6" t="inlineStr">
         <is>
           <t>29/08/2026</t>
         </is>
       </c>
-      <c r="H6" t="inlineStr">
+      <c r="L6" t="inlineStr">
         <is>
           <t>Demandes</t>
         </is>
       </c>
-      <c r="I6" t="inlineStr">
+      <c r="M6" t="inlineStr">
         <is>
           <t>Compteur partagé, sans doublon</t>
         </is>
@@ -5324,30 +5452,50 @@
       </c>
       <c r="D7" t="inlineStr">
         <is>
+          <t>Terminé</t>
+        </is>
+      </c>
+      <c r="E7" t="inlineStr">
+        <is>
+          <t>Terminé</t>
+        </is>
+      </c>
+      <c r="F7" t="inlineStr">
+        <is>
+          <t>Terminé</t>
+        </is>
+      </c>
+      <c r="G7" t="inlineStr">
+        <is>
+          <t>Terminé</t>
+        </is>
+      </c>
+      <c r="H7" t="inlineStr">
+        <is>
           <t>Moyen</t>
         </is>
       </c>
-      <c r="E7" t="inlineStr">
-        <is>
-          <t>DSI</t>
-        </is>
-      </c>
-      <c r="F7" t="inlineStr">
+      <c r="I7" t="inlineStr">
+        <is>
+          <t>DSI</t>
+        </is>
+      </c>
+      <c r="J7" t="inlineStr">
         <is>
           <t>28/08/2026</t>
         </is>
       </c>
-      <c r="G7" t="inlineStr">
+      <c r="K7" t="inlineStr">
         <is>
           <t>01/09/2026</t>
         </is>
       </c>
-      <c r="H7" t="inlineStr">
+      <c r="L7" t="inlineStr">
         <is>
           <t>Demandes</t>
         </is>
       </c>
-      <c r="I7" t="inlineStr">
+      <c r="M7" t="inlineStr">
         <is>
           <t>Demande créable sans montant</t>
         </is>
@@ -5371,30 +5519,50 @@
       </c>
       <c r="D8" t="inlineStr">
         <is>
+          <t>Terminé</t>
+        </is>
+      </c>
+      <c r="E8" t="inlineStr">
+        <is>
+          <t>Terminé</t>
+        </is>
+      </c>
+      <c r="F8" t="inlineStr">
+        <is>
+          <t>Terminé</t>
+        </is>
+      </c>
+      <c r="G8" t="inlineStr">
+        <is>
+          <t>Terminé</t>
+        </is>
+      </c>
+      <c r="H8" t="inlineStr">
+        <is>
           <t>Urgent</t>
         </is>
       </c>
-      <c r="E8" t="inlineStr">
-        <is>
-          <t>DSI</t>
-        </is>
-      </c>
-      <c r="F8" t="inlineStr">
+      <c r="I8" t="inlineStr">
+        <is>
+          <t>DSI</t>
+        </is>
+      </c>
+      <c r="J8" t="inlineStr">
         <is>
           <t>28/08/2026</t>
         </is>
       </c>
-      <c r="G8" t="inlineStr">
+      <c r="K8" t="inlineStr">
         <is>
           <t>30/08/2026</t>
         </is>
       </c>
-      <c r="H8" t="inlineStr">
+      <c r="L8" t="inlineStr">
         <is>
           <t>Fournisseurs</t>
         </is>
       </c>
-      <c r="I8" t="inlineStr">
+      <c r="M8" t="inlineStr">
         <is>
           <t>Nom, références, emplacement, WhatsApp, site</t>
         </is>
@@ -5418,30 +5586,50 @@
       </c>
       <c r="D9" t="inlineStr">
         <is>
+          <t>Terminé</t>
+        </is>
+      </c>
+      <c r="E9" t="inlineStr">
+        <is>
+          <t>Terminé</t>
+        </is>
+      </c>
+      <c r="F9" t="inlineStr">
+        <is>
+          <t>Terminé</t>
+        </is>
+      </c>
+      <c r="G9" t="inlineStr">
+        <is>
+          <t>Terminé</t>
+        </is>
+      </c>
+      <c r="H9" t="inlineStr">
+        <is>
           <t>Urgent</t>
         </is>
       </c>
-      <c r="E9" t="inlineStr">
-        <is>
-          <t>DSI</t>
-        </is>
-      </c>
-      <c r="F9" t="inlineStr">
+      <c r="I9" t="inlineStr">
+        <is>
+          <t>DSI</t>
+        </is>
+      </c>
+      <c r="J9" t="inlineStr">
         <is>
           <t>28/08/2026</t>
         </is>
       </c>
-      <c r="G9" t="inlineStr">
+      <c r="K9" t="inlineStr">
         <is>
           <t>30/08/2026</t>
         </is>
       </c>
-      <c r="H9" t="inlineStr">
+      <c r="L9" t="inlineStr">
         <is>
           <t>Fournisseurs</t>
         </is>
       </c>
-      <c r="I9" t="inlineStr">
+      <c r="M9" t="inlineStr">
         <is>
           <t>Aperçu, lignes invalides signalées</t>
         </is>
@@ -5465,30 +5653,50 @@
       </c>
       <c r="D10" t="inlineStr">
         <is>
+          <t>Terminé</t>
+        </is>
+      </c>
+      <c r="E10" t="inlineStr">
+        <is>
+          <t>Terminé</t>
+        </is>
+      </c>
+      <c r="F10" t="inlineStr">
+        <is>
+          <t>Terminé</t>
+        </is>
+      </c>
+      <c r="G10" t="inlineStr">
+        <is>
+          <t>Terminé</t>
+        </is>
+      </c>
+      <c r="H10" t="inlineStr">
+        <is>
           <t>Moyen</t>
         </is>
       </c>
-      <c r="E10" t="inlineStr">
-        <is>
-          <t>DSI</t>
-        </is>
-      </c>
-      <c r="F10" t="inlineStr">
+      <c r="I10" t="inlineStr">
+        <is>
+          <t>DSI</t>
+        </is>
+      </c>
+      <c r="J10" t="inlineStr">
         <is>
           <t>28/08/2026</t>
         </is>
       </c>
-      <c r="G10" t="inlineStr">
+      <c r="K10" t="inlineStr">
         <is>
           <t>30/08/2026</t>
         </is>
       </c>
-      <c r="H10" t="inlineStr">
+      <c r="L10" t="inlineStr">
         <is>
           <t>Fournisseurs</t>
         </is>
       </c>
-      <c r="I10" t="inlineStr">
+      <c r="M10" t="inlineStr">
         <is>
           <t>Excel, JSON, CSV</t>
         </is>
@@ -5512,30 +5720,50 @@
       </c>
       <c r="D11" t="inlineStr">
         <is>
+          <t>Terminé</t>
+        </is>
+      </c>
+      <c r="E11" t="inlineStr">
+        <is>
+          <t>Terminé</t>
+        </is>
+      </c>
+      <c r="F11" t="inlineStr">
+        <is>
+          <t>Terminé</t>
+        </is>
+      </c>
+      <c r="G11" t="inlineStr">
+        <is>
+          <t>Terminé</t>
+        </is>
+      </c>
+      <c r="H11" t="inlineStr">
+        <is>
           <t>Urgent</t>
         </is>
       </c>
-      <c r="E11" t="inlineStr">
-        <is>
-          <t>DSI</t>
-        </is>
-      </c>
-      <c r="F11" t="inlineStr">
+      <c r="I11" t="inlineStr">
+        <is>
+          <t>DSI</t>
+        </is>
+      </c>
+      <c r="J11" t="inlineStr">
         <is>
           <t>28/08/2026</t>
         </is>
       </c>
-      <c r="G11" t="inlineStr">
+      <c r="K11" t="inlineStr">
         <is>
           <t>31/08/2026</t>
         </is>
       </c>
-      <c r="H11" t="inlineStr">
+      <c r="L11" t="inlineStr">
         <is>
           <t>Négociation</t>
         </is>
       </c>
-      <c r="I11" t="inlineStr">
+      <c r="M11" t="inlineStr">
         <is>
           <t>Un prix par article et par fournisseur</t>
         </is>
@@ -5559,30 +5787,50 @@
       </c>
       <c r="D12" t="inlineStr">
         <is>
+          <t>Terminé</t>
+        </is>
+      </c>
+      <c r="E12" t="inlineStr">
+        <is>
+          <t>Terminé</t>
+        </is>
+      </c>
+      <c r="F12" t="inlineStr">
+        <is>
+          <t>Terminé</t>
+        </is>
+      </c>
+      <c r="G12" t="inlineStr">
+        <is>
+          <t>Terminé</t>
+        </is>
+      </c>
+      <c r="H12" t="inlineStr">
+        <is>
           <t>Urgent</t>
         </is>
       </c>
-      <c r="E12" t="inlineStr">
-        <is>
-          <t>DSI</t>
-        </is>
-      </c>
-      <c r="F12" t="inlineStr">
+      <c r="I12" t="inlineStr">
+        <is>
+          <t>DSI</t>
+        </is>
+      </c>
+      <c r="J12" t="inlineStr">
         <is>
           <t>28/08/2026</t>
         </is>
       </c>
-      <c r="G12" t="inlineStr">
+      <c r="K12" t="inlineStr">
         <is>
           <t>02/09/2026</t>
         </is>
       </c>
-      <c r="H12" t="inlineStr">
+      <c r="L12" t="inlineStr">
         <is>
           <t>Négociation</t>
         </is>
       </c>
-      <c r="I12" t="inlineStr">
+      <c r="M12" t="inlineStr">
         <is>
           <t>Seuil 0 = facultatif</t>
         </is>
@@ -5606,30 +5854,50 @@
       </c>
       <c r="D13" t="inlineStr">
         <is>
+          <t>Terminé</t>
+        </is>
+      </c>
+      <c r="E13" t="inlineStr">
+        <is>
+          <t>Terminé</t>
+        </is>
+      </c>
+      <c r="F13" t="inlineStr">
+        <is>
+          <t>Terminé</t>
+        </is>
+      </c>
+      <c r="G13" t="inlineStr">
+        <is>
+          <t>Terminé</t>
+        </is>
+      </c>
+      <c r="H13" t="inlineStr">
+        <is>
           <t>Urgent</t>
         </is>
       </c>
-      <c r="E13" t="inlineStr">
-        <is>
-          <t>DSI</t>
-        </is>
-      </c>
-      <c r="F13" t="inlineStr">
+      <c r="I13" t="inlineStr">
+        <is>
+          <t>DSI</t>
+        </is>
+      </c>
+      <c r="J13" t="inlineStr">
         <is>
           <t>28/08/2026</t>
         </is>
       </c>
-      <c r="G13" t="inlineStr">
+      <c r="K13" t="inlineStr">
         <is>
           <t>31/08/2026</t>
         </is>
       </c>
-      <c r="H13" t="inlineStr">
+      <c r="L13" t="inlineStr">
         <is>
           <t>Négociation</t>
         </is>
       </c>
-      <c r="I13" t="inlineStr">
+      <c r="M13" t="inlineStr">
         <is>
           <t>Comparaison fiable des offres</t>
         </is>
@@ -5653,30 +5921,50 @@
       </c>
       <c r="D14" t="inlineStr">
         <is>
+          <t>Terminé</t>
+        </is>
+      </c>
+      <c r="E14" t="inlineStr">
+        <is>
+          <t>Terminé</t>
+        </is>
+      </c>
+      <c r="F14" t="inlineStr">
+        <is>
+          <t>Terminé</t>
+        </is>
+      </c>
+      <c r="G14" t="inlineStr">
+        <is>
+          <t>Terminé</t>
+        </is>
+      </c>
+      <c r="H14" t="inlineStr">
+        <is>
           <t>Moyen</t>
         </is>
       </c>
-      <c r="E14" t="inlineStr">
-        <is>
-          <t>DSI</t>
-        </is>
-      </c>
-      <c r="F14" t="inlineStr">
+      <c r="I14" t="inlineStr">
+        <is>
+          <t>DSI</t>
+        </is>
+      </c>
+      <c r="J14" t="inlineStr">
         <is>
           <t>28/08/2026</t>
         </is>
       </c>
-      <c r="G14" t="inlineStr">
+      <c r="K14" t="inlineStr">
         <is>
           <t>31/08/2026</t>
         </is>
       </c>
-      <c r="H14" t="inlineStr">
+      <c r="L14" t="inlineStr">
         <is>
           <t>Négociation</t>
         </is>
       </c>
-      <c r="I14" t="inlineStr">
+      <c r="M14" t="inlineStr">
         <is>
           <t>Prix, délai, garantie, paiement</t>
         </is>
@@ -5700,30 +5988,50 @@
       </c>
       <c r="D15" t="inlineStr">
         <is>
+          <t>Terminé</t>
+        </is>
+      </c>
+      <c r="E15" t="inlineStr">
+        <is>
+          <t>Terminé</t>
+        </is>
+      </c>
+      <c r="F15" t="inlineStr">
+        <is>
+          <t>Terminé</t>
+        </is>
+      </c>
+      <c r="G15" t="inlineStr">
+        <is>
+          <t>Terminé</t>
+        </is>
+      </c>
+      <c r="H15" t="inlineStr">
+        <is>
           <t>Urgent</t>
         </is>
       </c>
-      <c r="E15" t="inlineStr">
-        <is>
-          <t>DSI</t>
-        </is>
-      </c>
-      <c r="F15" t="inlineStr">
+      <c r="I15" t="inlineStr">
+        <is>
+          <t>DSI</t>
+        </is>
+      </c>
+      <c r="J15" t="inlineStr">
         <is>
           <t>28/08/2026</t>
         </is>
       </c>
-      <c r="G15" t="inlineStr">
+      <c r="K15" t="inlineStr">
         <is>
           <t>31/08/2026</t>
         </is>
       </c>
-      <c r="H15" t="inlineStr">
+      <c r="L15" t="inlineStr">
         <is>
           <t>Négociation</t>
         </is>
       </c>
-      <c r="I15" t="inlineStr">
+      <c r="M15" t="inlineStr">
         <is>
           <t>Lecture seule, étape non bloquante</t>
         </is>
@@ -5747,30 +6055,50 @@
       </c>
       <c r="D16" t="inlineStr">
         <is>
+          <t>Terminé</t>
+        </is>
+      </c>
+      <c r="E16" t="inlineStr">
+        <is>
+          <t>Terminé</t>
+        </is>
+      </c>
+      <c r="F16" t="inlineStr">
+        <is>
+          <t>Terminé</t>
+        </is>
+      </c>
+      <c r="G16" t="inlineStr">
+        <is>
+          <t>Terminé</t>
+        </is>
+      </c>
+      <c r="H16" t="inlineStr">
+        <is>
           <t>Urgent</t>
         </is>
       </c>
-      <c r="E16" t="inlineStr">
-        <is>
-          <t>DSI</t>
-        </is>
-      </c>
-      <c r="F16" t="inlineStr">
+      <c r="I16" t="inlineStr">
+        <is>
+          <t>DSI</t>
+        </is>
+      </c>
+      <c r="J16" t="inlineStr">
         <is>
           <t>28/08/2026</t>
         </is>
       </c>
-      <c r="G16" t="inlineStr">
+      <c r="K16" t="inlineStr">
         <is>
           <t>01/09/2026</t>
         </is>
       </c>
-      <c r="H16" t="inlineStr">
+      <c r="L16" t="inlineStr">
         <is>
           <t>Validation</t>
         </is>
       </c>
-      <c r="I16" t="inlineStr">
+      <c r="M16" t="inlineStr">
         <is>
           <t>Motif obligatoire si refus</t>
         </is>
@@ -5794,30 +6122,50 @@
       </c>
       <c r="D17" t="inlineStr">
         <is>
+          <t>Terminé</t>
+        </is>
+      </c>
+      <c r="E17" t="inlineStr">
+        <is>
+          <t>Terminé</t>
+        </is>
+      </c>
+      <c r="F17" t="inlineStr">
+        <is>
+          <t>Terminé</t>
+        </is>
+      </c>
+      <c r="G17" t="inlineStr">
+        <is>
+          <t>Terminé</t>
+        </is>
+      </c>
+      <c r="H17" t="inlineStr">
+        <is>
           <t>Urgent</t>
         </is>
       </c>
-      <c r="E17" t="inlineStr">
-        <is>
-          <t>DSI</t>
-        </is>
-      </c>
-      <c r="F17" t="inlineStr">
+      <c r="I17" t="inlineStr">
+        <is>
+          <t>DSI</t>
+        </is>
+      </c>
+      <c r="J17" t="inlineStr">
         <is>
           <t>28/08/2026</t>
         </is>
       </c>
-      <c r="G17" t="inlineStr">
+      <c r="K17" t="inlineStr">
         <is>
           <t>01/09/2026</t>
         </is>
       </c>
-      <c r="H17" t="inlineStr">
+      <c r="L17" t="inlineStr">
         <is>
           <t>Commandes</t>
         </is>
       </c>
-      <c r="I17" t="inlineStr">
+      <c r="M17" t="inlineStr">
         <is>
           <t>Lignes aux prix négociés</t>
         </is>
@@ -5841,30 +6189,50 @@
       </c>
       <c r="D18" t="inlineStr">
         <is>
+          <t>Terminé</t>
+        </is>
+      </c>
+      <c r="E18" t="inlineStr">
+        <is>
+          <t>Terminé</t>
+        </is>
+      </c>
+      <c r="F18" t="inlineStr">
+        <is>
+          <t>Terminé</t>
+        </is>
+      </c>
+      <c r="G18" t="inlineStr">
+        <is>
+          <t>Terminé</t>
+        </is>
+      </c>
+      <c r="H18" t="inlineStr">
+        <is>
           <t>Moyen</t>
         </is>
       </c>
-      <c r="E18" t="inlineStr">
-        <is>
-          <t>DSI</t>
-        </is>
-      </c>
-      <c r="F18" t="inlineStr">
+      <c r="I18" t="inlineStr">
+        <is>
+          <t>DSI</t>
+        </is>
+      </c>
+      <c r="J18" t="inlineStr">
         <is>
           <t>28/08/2026</t>
         </is>
       </c>
-      <c r="G18" t="inlineStr">
+      <c r="K18" t="inlineStr">
         <is>
           <t>02/09/2026</t>
         </is>
       </c>
-      <c r="H18" t="inlineStr">
+      <c r="L18" t="inlineStr">
         <is>
           <t>Commandes</t>
         </is>
       </c>
-      <c r="I18" t="inlineStr">
+      <c r="M18" t="inlineStr">
         <is>
           <t>Cas des consultations en cours</t>
         </is>
@@ -5888,30 +6256,50 @@
       </c>
       <c r="D19" t="inlineStr">
         <is>
+          <t>Terminé</t>
+        </is>
+      </c>
+      <c r="E19" t="inlineStr">
+        <is>
+          <t>Terminé</t>
+        </is>
+      </c>
+      <c r="F19" t="inlineStr">
+        <is>
+          <t>Terminé</t>
+        </is>
+      </c>
+      <c r="G19" t="inlineStr">
+        <is>
+          <t>Terminé</t>
+        </is>
+      </c>
+      <c r="H19" t="inlineStr">
+        <is>
           <t>Urgent</t>
         </is>
       </c>
-      <c r="E19" t="inlineStr">
-        <is>
-          <t>DSI</t>
-        </is>
-      </c>
-      <c r="F19" t="inlineStr">
+      <c r="I19" t="inlineStr">
+        <is>
+          <t>DSI</t>
+        </is>
+      </c>
+      <c r="J19" t="inlineStr">
         <is>
           <t>28/08/2026</t>
         </is>
       </c>
-      <c r="G19" t="inlineStr">
+      <c r="K19" t="inlineStr">
         <is>
           <t>01/09/2026</t>
         </is>
       </c>
-      <c r="H19" t="inlineStr">
+      <c r="L19" t="inlineStr">
         <is>
           <t>Commandes</t>
         </is>
       </c>
-      <c r="I19" t="inlineStr">
+      <c r="M19" t="inlineStr">
         <is>
           <t>Clôture automatique si complète</t>
         </is>
@@ -5935,30 +6323,50 @@
       </c>
       <c r="D20" t="inlineStr">
         <is>
+          <t>Terminé</t>
+        </is>
+      </c>
+      <c r="E20" t="inlineStr">
+        <is>
+          <t>Terminé</t>
+        </is>
+      </c>
+      <c r="F20" t="inlineStr">
+        <is>
+          <t>Terminé</t>
+        </is>
+      </c>
+      <c r="G20" t="inlineStr">
+        <is>
+          <t>Terminé</t>
+        </is>
+      </c>
+      <c r="H20" t="inlineStr">
+        <is>
           <t>Urgent</t>
         </is>
       </c>
-      <c r="E20" t="inlineStr">
-        <is>
-          <t>DSI</t>
-        </is>
-      </c>
-      <c r="F20" t="inlineStr">
+      <c r="I20" t="inlineStr">
+        <is>
+          <t>DSI</t>
+        </is>
+      </c>
+      <c r="J20" t="inlineStr">
         <is>
           <t>28/08/2026</t>
         </is>
       </c>
-      <c r="G20" t="inlineStr">
+      <c r="K20" t="inlineStr">
         <is>
           <t>01/09/2026</t>
         </is>
       </c>
-      <c r="H20" t="inlineStr">
+      <c r="L20" t="inlineStr">
         <is>
           <t>Administration</t>
         </is>
       </c>
-      <c r="I20" t="inlineStr">
+      <c r="M20" t="inlineStr">
         <is>
           <t>Cascades et garde-fous</t>
         </is>
@@ -5982,30 +6390,50 @@
       </c>
       <c r="D21" t="inlineStr">
         <is>
+          <t>Terminé</t>
+        </is>
+      </c>
+      <c r="E21" t="inlineStr">
+        <is>
+          <t>Terminé</t>
+        </is>
+      </c>
+      <c r="F21" t="inlineStr">
+        <is>
+          <t>Terminé</t>
+        </is>
+      </c>
+      <c r="G21" t="inlineStr">
+        <is>
+          <t>Terminé</t>
+        </is>
+      </c>
+      <c r="H21" t="inlineStr">
+        <is>
           <t>Urgent</t>
         </is>
       </c>
-      <c r="E21" t="inlineStr">
-        <is>
-          <t>DSI</t>
-        </is>
-      </c>
-      <c r="F21" t="inlineStr">
+      <c r="I21" t="inlineStr">
+        <is>
+          <t>DSI</t>
+        </is>
+      </c>
+      <c r="J21" t="inlineStr">
         <is>
           <t>28/08/2026</t>
         </is>
       </c>
-      <c r="G21" t="inlineStr">
+      <c r="K21" t="inlineStr">
         <is>
           <t>02/09/2026</t>
         </is>
       </c>
-      <c r="H21" t="inlineStr">
+      <c r="L21" t="inlineStr">
         <is>
           <t>Alertes</t>
         </is>
       </c>
-      <c r="I21" t="inlineStr">
+      <c r="M21" t="inlineStr">
         <is>
           <t>Validation et réception, anti-doublon</t>
         </is>
@@ -6029,30 +6457,50 @@
       </c>
       <c r="D22" t="inlineStr">
         <is>
+          <t>Terminé</t>
+        </is>
+      </c>
+      <c r="E22" t="inlineStr">
+        <is>
+          <t>Terminé</t>
+        </is>
+      </c>
+      <c r="F22" t="inlineStr">
+        <is>
+          <t>Terminé</t>
+        </is>
+      </c>
+      <c r="G22" t="inlineStr">
+        <is>
+          <t>Terminé</t>
+        </is>
+      </c>
+      <c r="H22" t="inlineStr">
+        <is>
           <t>Moyen</t>
         </is>
       </c>
-      <c r="E22" t="inlineStr">
-        <is>
-          <t>DSI</t>
-        </is>
-      </c>
-      <c r="F22" t="inlineStr">
+      <c r="I22" t="inlineStr">
+        <is>
+          <t>DSI</t>
+        </is>
+      </c>
+      <c r="J22" t="inlineStr">
         <is>
           <t>28/08/2026</t>
         </is>
       </c>
-      <c r="G22" t="inlineStr">
+      <c r="K22" t="inlineStr">
         <is>
           <t>02/09/2026</t>
         </is>
       </c>
-      <c r="H22" t="inlineStr">
+      <c r="L22" t="inlineStr">
         <is>
           <t>Alertes</t>
         </is>
       </c>
-      <c r="I22" t="inlineStr">
+      <c r="M22" t="inlineStr">
         <is>
           <t>Vue immédiate des retards</t>
         </is>
@@ -6076,30 +6524,50 @@
       </c>
       <c r="D23" t="inlineStr">
         <is>
+          <t>Terminé</t>
+        </is>
+      </c>
+      <c r="E23" t="inlineStr">
+        <is>
+          <t>Terminé</t>
+        </is>
+      </c>
+      <c r="F23" t="inlineStr">
+        <is>
+          <t>Terminé</t>
+        </is>
+      </c>
+      <c r="G23" t="inlineStr">
+        <is>
+          <t>Terminé</t>
+        </is>
+      </c>
+      <c r="H23" t="inlineStr">
+        <is>
           <t>Moyen</t>
         </is>
       </c>
-      <c r="E23" t="inlineStr">
-        <is>
-          <t>DSI</t>
-        </is>
-      </c>
-      <c r="F23" t="inlineStr">
+      <c r="I23" t="inlineStr">
+        <is>
+          <t>DSI</t>
+        </is>
+      </c>
+      <c r="J23" t="inlineStr">
         <is>
           <t>28/08/2026</t>
         </is>
       </c>
-      <c r="G23" t="inlineStr">
+      <c r="K23" t="inlineStr">
         <is>
           <t>02/09/2026</t>
         </is>
       </c>
-      <c r="H23" t="inlineStr">
+      <c r="L23" t="inlineStr">
         <is>
           <t>Alertes</t>
         </is>
       </c>
-      <c r="I23" t="inlineStr">
+      <c r="M23" t="inlineStr">
         <is>
           <t>Avec son de secours si bloqué</t>
         </is>
@@ -6123,30 +6591,50 @@
       </c>
       <c r="D24" t="inlineStr">
         <is>
+          <t>Terminé</t>
+        </is>
+      </c>
+      <c r="E24" t="inlineStr">
+        <is>
+          <t>Terminé</t>
+        </is>
+      </c>
+      <c r="F24" t="inlineStr">
+        <is>
+          <t>Terminé</t>
+        </is>
+      </c>
+      <c r="G24" t="inlineStr">
+        <is>
+          <t>Terminé</t>
+        </is>
+      </c>
+      <c r="H24" t="inlineStr">
+        <is>
           <t>Moyen</t>
         </is>
       </c>
-      <c r="E24" t="inlineStr">
-        <is>
-          <t>DSI</t>
-        </is>
-      </c>
-      <c r="F24" t="inlineStr">
+      <c r="I24" t="inlineStr">
+        <is>
+          <t>DSI</t>
+        </is>
+      </c>
+      <c r="J24" t="inlineStr">
         <is>
           <t>28/08/2026</t>
         </is>
       </c>
-      <c r="G24" t="inlineStr">
+      <c r="K24" t="inlineStr">
         <is>
           <t>02/09/2026</t>
         </is>
       </c>
-      <c r="H24" t="inlineStr">
+      <c r="L24" t="inlineStr">
         <is>
           <t>Alertes</t>
         </is>
       </c>
-      <c r="I24" t="inlineStr">
+      <c r="M24" t="inlineStr">
         <is>
           <t>15 s, maximum 10 répétitions</t>
         </is>
@@ -6170,30 +6658,50 @@
       </c>
       <c r="D25" t="inlineStr">
         <is>
+          <t>Terminé</t>
+        </is>
+      </c>
+      <c r="E25" t="inlineStr">
+        <is>
+          <t>Terminé</t>
+        </is>
+      </c>
+      <c r="F25" t="inlineStr">
+        <is>
+          <t>Terminé</t>
+        </is>
+      </c>
+      <c r="G25" t="inlineStr">
+        <is>
+          <t>Terminé</t>
+        </is>
+      </c>
+      <c r="H25" t="inlineStr">
+        <is>
           <t>Moyen</t>
         </is>
       </c>
-      <c r="E25" t="inlineStr">
-        <is>
-          <t>DSI</t>
-        </is>
-      </c>
-      <c r="F25" t="inlineStr">
+      <c r="I25" t="inlineStr">
+        <is>
+          <t>DSI</t>
+        </is>
+      </c>
+      <c r="J25" t="inlineStr">
         <is>
           <t>28/08/2026</t>
         </is>
       </c>
-      <c r="G25" t="inlineStr">
+      <c r="K25" t="inlineStr">
         <is>
           <t>02/09/2026</t>
         </is>
       </c>
-      <c r="H25" t="inlineStr">
+      <c r="L25" t="inlineStr">
         <is>
           <t>Alertes</t>
         </is>
       </c>
-      <c r="I25" t="inlineStr">
+      <c r="M25" t="inlineStr">
         <is>
           <t>Actives onglet en arrière-plan</t>
         </is>
@@ -6217,30 +6725,50 @@
       </c>
       <c r="D26" t="inlineStr">
         <is>
+          <t>Terminé</t>
+        </is>
+      </c>
+      <c r="E26" t="inlineStr">
+        <is>
+          <t>Terminé</t>
+        </is>
+      </c>
+      <c r="F26" t="inlineStr">
+        <is>
+          <t>Terminé</t>
+        </is>
+      </c>
+      <c r="G26" t="inlineStr">
+        <is>
+          <t>Terminé</t>
+        </is>
+      </c>
+      <c r="H26" t="inlineStr">
+        <is>
           <t>Moyen</t>
         </is>
       </c>
-      <c r="E26" t="inlineStr">
-        <is>
-          <t>DSI</t>
-        </is>
-      </c>
-      <c r="F26" t="inlineStr">
+      <c r="I26" t="inlineStr">
+        <is>
+          <t>DSI</t>
+        </is>
+      </c>
+      <c r="J26" t="inlineStr">
         <is>
           <t>28/08/2026</t>
         </is>
       </c>
-      <c r="G26" t="inlineStr">
+      <c r="K26" t="inlineStr">
         <is>
           <t>02/09/2026</t>
         </is>
       </c>
-      <c r="H26" t="inlineStr">
+      <c r="L26" t="inlineStr">
         <is>
           <t>Alertes</t>
         </is>
       </c>
-      <c r="I26" t="inlineStr">
+      <c r="M26" t="inlineStr">
         <is>
           <t>Secours si le son est coupé</t>
         </is>
@@ -6264,30 +6792,50 @@
       </c>
       <c r="D27" t="inlineStr">
         <is>
+          <t>Terminé</t>
+        </is>
+      </c>
+      <c r="E27" t="inlineStr">
+        <is>
+          <t>Terminé</t>
+        </is>
+      </c>
+      <c r="F27" t="inlineStr">
+        <is>
+          <t>Terminé</t>
+        </is>
+      </c>
+      <c r="G27" t="inlineStr">
+        <is>
+          <t>Terminé</t>
+        </is>
+      </c>
+      <c r="H27" t="inlineStr">
+        <is>
           <t>Urgent</t>
         </is>
       </c>
-      <c r="E27" t="inlineStr">
-        <is>
-          <t>DSI</t>
-        </is>
-      </c>
-      <c r="F27" t="inlineStr">
+      <c r="I27" t="inlineStr">
+        <is>
+          <t>DSI</t>
+        </is>
+      </c>
+      <c r="J27" t="inlineStr">
         <is>
           <t>28/08/2026</t>
         </is>
       </c>
-      <c r="G27" t="inlineStr">
+      <c r="K27" t="inlineStr">
         <is>
           <t>02/09/2026</t>
         </is>
       </c>
-      <c r="H27" t="inlineStr">
+      <c r="L27" t="inlineStr">
         <is>
           <t>Documents</t>
         </is>
       </c>
-      <c r="I27" t="inlineStr">
+      <c r="M27" t="inlineStr">
         <is>
           <t>Colonnes de prix vides à compléter</t>
         </is>
@@ -6311,30 +6859,50 @@
       </c>
       <c r="D28" t="inlineStr">
         <is>
+          <t>Terminé</t>
+        </is>
+      </c>
+      <c r="E28" t="inlineStr">
+        <is>
+          <t>Terminé</t>
+        </is>
+      </c>
+      <c r="F28" t="inlineStr">
+        <is>
+          <t>Terminé</t>
+        </is>
+      </c>
+      <c r="G28" t="inlineStr">
+        <is>
+          <t>Terminé</t>
+        </is>
+      </c>
+      <c r="H28" t="inlineStr">
+        <is>
           <t>Urgent</t>
         </is>
       </c>
-      <c r="E28" t="inlineStr">
-        <is>
-          <t>DSI</t>
-        </is>
-      </c>
-      <c r="F28" t="inlineStr">
+      <c r="I28" t="inlineStr">
+        <is>
+          <t>DSI</t>
+        </is>
+      </c>
+      <c r="J28" t="inlineStr">
         <is>
           <t>28/08/2026</t>
         </is>
       </c>
-      <c r="G28" t="inlineStr">
+      <c r="K28" t="inlineStr">
         <is>
           <t>01/09/2026</t>
         </is>
       </c>
-      <c r="H28" t="inlineStr">
+      <c r="L28" t="inlineStr">
         <is>
           <t>Documents</t>
         </is>
       </c>
-      <c r="I28" t="inlineStr">
+      <c r="M28" t="inlineStr">
         <is>
           <t>jsPDF, repli impression</t>
         </is>
@@ -6358,30 +6926,50 @@
       </c>
       <c r="D29" t="inlineStr">
         <is>
+          <t>Terminé</t>
+        </is>
+      </c>
+      <c r="E29" t="inlineStr">
+        <is>
+          <t>Terminé</t>
+        </is>
+      </c>
+      <c r="F29" t="inlineStr">
+        <is>
+          <t>Terminé</t>
+        </is>
+      </c>
+      <c r="G29" t="inlineStr">
+        <is>
+          <t>Terminé</t>
+        </is>
+      </c>
+      <c r="H29" t="inlineStr">
+        <is>
           <t>Moyen</t>
         </is>
       </c>
-      <c r="E29" t="inlineStr">
-        <is>
-          <t>DSI</t>
-        </is>
-      </c>
-      <c r="F29" t="inlineStr">
+      <c r="I29" t="inlineStr">
+        <is>
+          <t>DSI</t>
+        </is>
+      </c>
+      <c r="J29" t="inlineStr">
         <is>
           <t>28/08/2026</t>
         </is>
       </c>
-      <c r="G29" t="inlineStr">
+      <c r="K29" t="inlineStr">
         <is>
           <t>01/09/2026</t>
         </is>
       </c>
-      <c r="H29" t="inlineStr">
+      <c r="L29" t="inlineStr">
         <is>
           <t>Documents</t>
         </is>
       </c>
-      <c r="I29" t="inlineStr">
+      <c r="M29" t="inlineStr">
         <is>
           <t>Comparaison incluse</t>
         </is>
@@ -6405,30 +6993,50 @@
       </c>
       <c r="D30" t="inlineStr">
         <is>
+          <t>Terminé</t>
+        </is>
+      </c>
+      <c r="E30" t="inlineStr">
+        <is>
+          <t>Terminé</t>
+        </is>
+      </c>
+      <c r="F30" t="inlineStr">
+        <is>
+          <t>Terminé</t>
+        </is>
+      </c>
+      <c r="G30" t="inlineStr">
+        <is>
+          <t>Terminé</t>
+        </is>
+      </c>
+      <c r="H30" t="inlineStr">
+        <is>
           <t>Moyen</t>
         </is>
       </c>
-      <c r="E30" t="inlineStr">
+      <c r="I30" t="inlineStr">
         <is>
           <t>Direction</t>
         </is>
       </c>
-      <c r="F30" t="inlineStr">
+      <c r="J30" t="inlineStr">
         <is>
           <t>28/08/2026</t>
         </is>
       </c>
-      <c r="G30" t="inlineStr">
+      <c r="K30" t="inlineStr">
         <is>
           <t>02/09/2026</t>
         </is>
       </c>
-      <c r="H30" t="inlineStr">
+      <c r="L30" t="inlineStr">
         <is>
           <t>Documents</t>
         </is>
       </c>
-      <c r="I30" t="inlineStr">
+      <c r="M30" t="inlineStr">
         <is>
           <t>Site, impressions, PDF, favicon</t>
         </is>
@@ -6452,30 +7060,50 @@
       </c>
       <c r="D31" t="inlineStr">
         <is>
+          <t>Terminé</t>
+        </is>
+      </c>
+      <c r="E31" t="inlineStr">
+        <is>
+          <t>Terminé</t>
+        </is>
+      </c>
+      <c r="F31" t="inlineStr">
+        <is>
+          <t>Terminé</t>
+        </is>
+      </c>
+      <c r="G31" t="inlineStr">
+        <is>
+          <t>Terminé</t>
+        </is>
+      </c>
+      <c r="H31" t="inlineStr">
+        <is>
           <t>Urgent</t>
         </is>
       </c>
-      <c r="E31" t="inlineStr">
-        <is>
-          <t>DSI</t>
-        </is>
-      </c>
-      <c r="F31" t="inlineStr">
+      <c r="I31" t="inlineStr">
+        <is>
+          <t>DSI</t>
+        </is>
+      </c>
+      <c r="J31" t="inlineStr">
         <is>
           <t>28/08/2026</t>
         </is>
       </c>
-      <c r="G31" t="inlineStr">
+      <c r="K31" t="inlineStr">
         <is>
           <t>02/09/2026</t>
         </is>
       </c>
-      <c r="H31" t="inlineStr">
+      <c r="L31" t="inlineStr">
         <is>
           <t>Données</t>
         </is>
       </c>
-      <c r="I31" t="inlineStr">
+      <c r="M31" t="inlineStr">
         <is>
           <t>Partage entre tous les postes</t>
         </is>
@@ -6499,30 +7127,50 @@
       </c>
       <c r="D32" t="inlineStr">
         <is>
+          <t>Terminé</t>
+        </is>
+      </c>
+      <c r="E32" t="inlineStr">
+        <is>
+          <t>Terminé</t>
+        </is>
+      </c>
+      <c r="F32" t="inlineStr">
+        <is>
+          <t>Terminé</t>
+        </is>
+      </c>
+      <c r="G32" t="inlineStr">
+        <is>
+          <t>Terminé</t>
+        </is>
+      </c>
+      <c r="H32" t="inlineStr">
+        <is>
           <t>Urgent</t>
         </is>
       </c>
-      <c r="E32" t="inlineStr">
-        <is>
-          <t>DSI</t>
-        </is>
-      </c>
-      <c r="F32" t="inlineStr">
+      <c r="I32" t="inlineStr">
+        <is>
+          <t>DSI</t>
+        </is>
+      </c>
+      <c r="J32" t="inlineStr">
         <is>
           <t>28/08/2026</t>
         </is>
       </c>
-      <c r="G32" t="inlineStr">
+      <c r="K32" t="inlineStr">
         <is>
           <t>02/09/2026</t>
         </is>
       </c>
-      <c r="H32" t="inlineStr">
+      <c r="L32" t="inlineStr">
         <is>
           <t>Données</t>
         </is>
       </c>
-      <c r="I32" t="inlineStr">
+      <c r="M32" t="inlineStr">
         <is>
           <t>Le serveur fait foi au démarrage</t>
         </is>
@@ -6546,30 +7194,50 @@
       </c>
       <c r="D33" t="inlineStr">
         <is>
+          <t>Terminé</t>
+        </is>
+      </c>
+      <c r="E33" t="inlineStr">
+        <is>
+          <t>Terminé</t>
+        </is>
+      </c>
+      <c r="F33" t="inlineStr">
+        <is>
+          <t>Terminé</t>
+        </is>
+      </c>
+      <c r="G33" t="inlineStr">
+        <is>
+          <t>Terminé</t>
+        </is>
+      </c>
+      <c r="H33" t="inlineStr">
+        <is>
           <t>Moyen</t>
         </is>
       </c>
-      <c r="E33" t="inlineStr">
-        <is>
-          <t>DSI</t>
-        </is>
-      </c>
-      <c r="F33" t="inlineStr">
+      <c r="I33" t="inlineStr">
+        <is>
+          <t>DSI</t>
+        </is>
+      </c>
+      <c r="J33" t="inlineStr">
         <is>
           <t>28/08/2026</t>
         </is>
       </c>
-      <c r="G33" t="inlineStr">
+      <c r="K33" t="inlineStr">
         <is>
           <t>02/09/2026</t>
         </is>
       </c>
-      <c r="H33" t="inlineStr">
+      <c r="L33" t="inlineStr">
         <is>
           <t>Pilotage</t>
         </is>
       </c>
-      <c r="I33" t="inlineStr">
+      <c r="M33" t="inlineStr">
         <is>
           <t>Achats 12 mois, répartition, top 5</t>
         </is>
@@ -6593,30 +7261,50 @@
       </c>
       <c r="D34" t="inlineStr">
         <is>
+          <t>Terminé</t>
+        </is>
+      </c>
+      <c r="E34" t="inlineStr">
+        <is>
+          <t>Terminé</t>
+        </is>
+      </c>
+      <c r="F34" t="inlineStr">
+        <is>
+          <t>Terminé</t>
+        </is>
+      </c>
+      <c r="G34" t="inlineStr">
+        <is>
+          <t>Terminé</t>
+        </is>
+      </c>
+      <c r="H34" t="inlineStr">
+        <is>
           <t>Urgent</t>
         </is>
       </c>
-      <c r="E34" t="inlineStr">
-        <is>
-          <t>DSI</t>
-        </is>
-      </c>
-      <c r="F34" t="inlineStr">
+      <c r="I34" t="inlineStr">
+        <is>
+          <t>DSI</t>
+        </is>
+      </c>
+      <c r="J34" t="inlineStr">
         <is>
           <t>28/08/2026</t>
         </is>
       </c>
-      <c r="G34" t="inlineStr">
+      <c r="K34" t="inlineStr">
         <is>
           <t>02/09/2026</t>
         </is>
       </c>
-      <c r="H34" t="inlineStr">
+      <c r="L34" t="inlineStr">
         <is>
           <t>Qualité</t>
         </is>
       </c>
-      <c r="I34" t="inlineStr">
+      <c r="M34" t="inlineStr">
         <is>
           <t>13 séries, exécutées avant publication</t>
         </is>
@@ -6640,30 +7328,50 @@
       </c>
       <c r="D35" t="inlineStr">
         <is>
+          <t>Terminé</t>
+        </is>
+      </c>
+      <c r="E35" t="inlineStr">
+        <is>
+          <t>Terminé</t>
+        </is>
+      </c>
+      <c r="F35" t="inlineStr">
+        <is>
+          <t>Terminé</t>
+        </is>
+      </c>
+      <c r="G35" t="inlineStr">
+        <is>
+          <t>Terminé</t>
+        </is>
+      </c>
+      <c r="H35" t="inlineStr">
+        <is>
           <t>Urgent</t>
         </is>
       </c>
-      <c r="E35" t="inlineStr">
-        <is>
-          <t>DSI</t>
-        </is>
-      </c>
-      <c r="F35" t="inlineStr">
+      <c r="I35" t="inlineStr">
+        <is>
+          <t>DSI</t>
+        </is>
+      </c>
+      <c r="J35" t="inlineStr">
         <is>
           <t>28/08/2026</t>
         </is>
       </c>
-      <c r="G35" t="inlineStr">
+      <c r="K35" t="inlineStr">
         <is>
           <t>02/09/2026</t>
         </is>
       </c>
-      <c r="H35" t="inlineStr">
+      <c r="L35" t="inlineStr">
         <is>
           <t>Déploiement</t>
         </is>
       </c>
-      <c r="I35" t="inlineStr">
+      <c r="M35" t="inlineStr">
         <is>
           <t>Une commande : scripts/publish.mjs</t>
         </is>
@@ -6687,30 +7395,50 @@
       </c>
       <c r="D36" t="inlineStr">
         <is>
+          <t>Terminé</t>
+        </is>
+      </c>
+      <c r="E36" t="inlineStr">
+        <is>
+          <t>Terminé</t>
+        </is>
+      </c>
+      <c r="F36" t="inlineStr">
+        <is>
+          <t>Terminé</t>
+        </is>
+      </c>
+      <c r="G36" t="inlineStr">
+        <is>
+          <t>Terminé</t>
+        </is>
+      </c>
+      <c r="H36" t="inlineStr">
+        <is>
           <t>Moyen</t>
         </is>
       </c>
-      <c r="E36" t="inlineStr">
-        <is>
-          <t>DSI</t>
-        </is>
-      </c>
-      <c r="F36" t="inlineStr">
+      <c r="I36" t="inlineStr">
+        <is>
+          <t>DSI</t>
+        </is>
+      </c>
+      <c r="J36" t="inlineStr">
         <is>
           <t>28/08/2026</t>
         </is>
       </c>
-      <c r="G36" t="inlineStr">
+      <c r="K36" t="inlineStr">
         <is>
           <t>02/09/2026</t>
         </is>
       </c>
-      <c r="H36" t="inlineStr">
+      <c r="L36" t="inlineStr">
         <is>
           <t>Documentation</t>
         </is>
       </c>
-      <c r="I36" t="inlineStr">
+      <c r="M36" t="inlineStr">
         <is>
           <t>PDF et Word, 14 et 4 pages</t>
         </is>
@@ -6734,30 +7462,50 @@
       </c>
       <c r="D37" t="inlineStr">
         <is>
+          <t>Terminé</t>
+        </is>
+      </c>
+      <c r="E37" t="inlineStr">
+        <is>
+          <t>En cours</t>
+        </is>
+      </c>
+      <c r="F37" t="inlineStr">
+        <is>
+          <t>Pas commencé</t>
+        </is>
+      </c>
+      <c r="G37" t="inlineStr">
+        <is>
+          <t>Pas commencé</t>
+        </is>
+      </c>
+      <c r="H37" t="inlineStr">
+        <is>
           <t>Urgent</t>
         </is>
       </c>
-      <c r="E37" t="inlineStr">
+      <c r="I37" t="inlineStr">
         <is>
           <t>Direction</t>
         </is>
       </c>
-      <c r="F37" t="inlineStr">
+      <c r="J37" t="inlineStr">
         <is>
           <t>28/08/2026</t>
         </is>
       </c>
-      <c r="G37" t="inlineStr">
+      <c r="K37" t="inlineStr">
         <is>
           <t>05/09/2026</t>
         </is>
       </c>
-      <c r="H37" t="inlineStr">
+      <c r="L37" t="inlineStr">
         <is>
           <t>Qualité</t>
         </is>
       </c>
-      <c r="I37" t="inlineStr">
+      <c r="M37" t="inlineStr">
         <is>
           <t>Retours des utilisateurs finaux</t>
         </is>
@@ -6781,30 +7529,50 @@
       </c>
       <c r="D38" t="inlineStr">
         <is>
+          <t>En cours</t>
+        </is>
+      </c>
+      <c r="E38" t="inlineStr">
+        <is>
+          <t>Pas commencé</t>
+        </is>
+      </c>
+      <c r="F38" t="inlineStr">
+        <is>
+          <t>Pas commencé</t>
+        </is>
+      </c>
+      <c r="G38" t="inlineStr">
+        <is>
+          <t>Pas commencé</t>
+        </is>
+      </c>
+      <c r="H38" t="inlineStr">
+        <is>
           <t>Urgent</t>
         </is>
       </c>
-      <c r="E38" t="inlineStr">
-        <is>
-          <t>DSI</t>
-        </is>
-      </c>
-      <c r="F38" t="inlineStr">
+      <c r="I38" t="inlineStr">
+        <is>
+          <t>DSI</t>
+        </is>
+      </c>
+      <c r="J38" t="inlineStr">
         <is>
           <t>28/08/2026</t>
         </is>
       </c>
-      <c r="G38" t="inlineStr">
+      <c r="K38" t="inlineStr">
         <is>
           <t>09/09/2026</t>
         </is>
       </c>
-      <c r="H38" t="inlineStr">
+      <c r="L38" t="inlineStr">
         <is>
           <t>Sécurité</t>
         </is>
       </c>
-      <c r="I38" t="inlineStr">
+      <c r="M38" t="inlineStr">
         <is>
           <t>Restreindre par rôle avant généralisation</t>
         </is>
@@ -6828,30 +7596,50 @@
       </c>
       <c r="D39" t="inlineStr">
         <is>
+          <t>En cours</t>
+        </is>
+      </c>
+      <c r="E39" t="inlineStr">
+        <is>
+          <t>Pas commencé</t>
+        </is>
+      </c>
+      <c r="F39" t="inlineStr">
+        <is>
+          <t>Pas commencé</t>
+        </is>
+      </c>
+      <c r="G39" t="inlineStr">
+        <is>
+          <t>Pas commencé</t>
+        </is>
+      </c>
+      <c r="H39" t="inlineStr">
+        <is>
           <t>Urgent</t>
         </is>
       </c>
-      <c r="E39" t="inlineStr">
-        <is>
-          <t>DSI</t>
-        </is>
-      </c>
-      <c r="F39" t="inlineStr">
+      <c r="I39" t="inlineStr">
+        <is>
+          <t>DSI</t>
+        </is>
+      </c>
+      <c r="J39" t="inlineStr">
         <is>
           <t>28/08/2026</t>
         </is>
       </c>
-      <c r="G39" t="inlineStr">
+      <c r="K39" t="inlineStr">
         <is>
           <t>12/09/2026</t>
         </is>
       </c>
-      <c r="H39" t="inlineStr">
+      <c r="L39" t="inlineStr">
         <is>
           <t>Sécurité</t>
         </is>
       </c>
-      <c r="I39" t="inlineStr">
+      <c r="M39" t="inlineStr">
         <is>
           <t>Qui a supprimé/modifié quoi et quand</t>
         </is>
@@ -6875,26 +7663,46 @@
       </c>
       <c r="D40" t="inlineStr">
         <is>
+          <t>Pas commencé</t>
+        </is>
+      </c>
+      <c r="E40" t="inlineStr">
+        <is>
+          <t>Pas commencé</t>
+        </is>
+      </c>
+      <c r="F40" t="inlineStr">
+        <is>
+          <t>Pas commencé</t>
+        </is>
+      </c>
+      <c r="G40" t="inlineStr">
+        <is>
+          <t>Pas commencé</t>
+        </is>
+      </c>
+      <c r="H40" t="inlineStr">
+        <is>
           <t>Urgent</t>
         </is>
       </c>
-      <c r="E40" t="inlineStr">
-        <is>
-          <t>DSI</t>
-        </is>
-      </c>
-      <c r="F40" t="inlineStr"/>
-      <c r="G40" t="inlineStr">
+      <c r="I40" t="inlineStr">
+        <is>
+          <t>DSI</t>
+        </is>
+      </c>
+      <c r="J40" t="inlineStr"/>
+      <c r="K40" t="inlineStr">
         <is>
           <t>19/09/2026</t>
         </is>
       </c>
-      <c r="H40" t="inlineStr">
+      <c r="L40" t="inlineStr">
         <is>
           <t>Sécurité</t>
         </is>
       </c>
-      <c r="I40" t="inlineStr">
+      <c r="M40" t="inlineStr">
         <is>
           <t>Migration vers Supabase Auth</t>
         </is>
@@ -6918,26 +7726,46 @@
       </c>
       <c r="D41" t="inlineStr">
         <is>
+          <t>Pas commencé</t>
+        </is>
+      </c>
+      <c r="E41" t="inlineStr">
+        <is>
+          <t>Pas commencé</t>
+        </is>
+      </c>
+      <c r="F41" t="inlineStr">
+        <is>
+          <t>Pas commencé</t>
+        </is>
+      </c>
+      <c r="G41" t="inlineStr">
+        <is>
+          <t>Pas commencé</t>
+        </is>
+      </c>
+      <c r="H41" t="inlineStr">
+        <is>
           <t>Moyen</t>
         </is>
       </c>
-      <c r="E41" t="inlineStr">
-        <is>
-          <t>DSI</t>
-        </is>
-      </c>
-      <c r="F41" t="inlineStr"/>
-      <c r="G41" t="inlineStr">
+      <c r="I41" t="inlineStr">
+        <is>
+          <t>DSI</t>
+        </is>
+      </c>
+      <c r="J41" t="inlineStr"/>
+      <c r="K41" t="inlineStr">
         <is>
           <t>26/09/2026</t>
         </is>
       </c>
-      <c r="H41" t="inlineStr">
+      <c r="L41" t="inlineStr">
         <is>
           <t>Alertes</t>
         </is>
       </c>
-      <c r="I41" t="inlineStr">
+      <c r="M41" t="inlineStr">
         <is>
           <t>Réduction des délais de réponse</t>
         </is>
@@ -6961,26 +7789,46 @@
       </c>
       <c r="D42" t="inlineStr">
         <is>
+          <t>Pas commencé</t>
+        </is>
+      </c>
+      <c r="E42" t="inlineStr">
+        <is>
+          <t>Pas commencé</t>
+        </is>
+      </c>
+      <c r="F42" t="inlineStr">
+        <is>
+          <t>Pas commencé</t>
+        </is>
+      </c>
+      <c r="G42" t="inlineStr">
+        <is>
+          <t>Pas commencé</t>
+        </is>
+      </c>
+      <c r="H42" t="inlineStr">
+        <is>
           <t>Moyen</t>
         </is>
       </c>
-      <c r="E42" t="inlineStr">
+      <c r="I42" t="inlineStr">
         <is>
           <t>Direction</t>
         </is>
       </c>
-      <c r="F42" t="inlineStr"/>
-      <c r="G42" t="inlineStr">
+      <c r="J42" t="inlineStr"/>
+      <c r="K42" t="inlineStr">
         <is>
           <t>10/10/2026</t>
         </is>
       </c>
-      <c r="H42" t="inlineStr">
+      <c r="L42" t="inlineStr">
         <is>
           <t>Pilotage</t>
         </is>
       </c>
-      <c r="I42" t="inlineStr">
+      <c r="M42" t="inlineStr">
         <is>
           <t>Pilotage financier</t>
         </is>
@@ -7004,26 +7852,46 @@
       </c>
       <c r="D43" t="inlineStr">
         <is>
+          <t>Pas commencé</t>
+        </is>
+      </c>
+      <c r="E43" t="inlineStr">
+        <is>
+          <t>Pas commencé</t>
+        </is>
+      </c>
+      <c r="F43" t="inlineStr">
+        <is>
+          <t>Pas commencé</t>
+        </is>
+      </c>
+      <c r="G43" t="inlineStr">
+        <is>
+          <t>Pas commencé</t>
+        </is>
+      </c>
+      <c r="H43" t="inlineStr">
+        <is>
           <t>Faible</t>
         </is>
       </c>
-      <c r="E43" t="inlineStr">
-        <is>
-          <t>DSI</t>
-        </is>
-      </c>
-      <c r="F43" t="inlineStr"/>
-      <c r="G43" t="inlineStr">
+      <c r="I43" t="inlineStr">
+        <is>
+          <t>DSI</t>
+        </is>
+      </c>
+      <c r="J43" t="inlineStr"/>
+      <c r="K43" t="inlineStr">
         <is>
           <t>24/10/2026</t>
         </is>
       </c>
-      <c r="H43" t="inlineStr">
+      <c r="L43" t="inlineStr">
         <is>
           <t>Fournisseurs</t>
         </is>
       </c>
-      <c r="I43" t="inlineStr">
+      <c r="M43" t="inlineStr">
         <is>
           <t>Productivité sur les consultations</t>
         </is>
@@ -7047,26 +7915,46 @@
       </c>
       <c r="D44" t="inlineStr">
         <is>
+          <t>Pas commencé</t>
+        </is>
+      </c>
+      <c r="E44" t="inlineStr">
+        <is>
+          <t>Pas commencé</t>
+        </is>
+      </c>
+      <c r="F44" t="inlineStr">
+        <is>
+          <t>Pas commencé</t>
+        </is>
+      </c>
+      <c r="G44" t="inlineStr">
+        <is>
+          <t>Pas commencé</t>
+        </is>
+      </c>
+      <c r="H44" t="inlineStr">
+        <is>
           <t>Faible</t>
         </is>
       </c>
-      <c r="E44" t="inlineStr">
+      <c r="I44" t="inlineStr">
         <is>
           <t>Logistique</t>
         </is>
       </c>
-      <c r="F44" t="inlineStr"/>
-      <c r="G44" t="inlineStr">
+      <c r="J44" t="inlineStr"/>
+      <c r="K44" t="inlineStr">
         <is>
           <t>31/10/2026</t>
         </is>
       </c>
-      <c r="H44" t="inlineStr">
+      <c r="L44" t="inlineStr">
         <is>
           <t>Pilotage</t>
         </is>
       </c>
-      <c r="I44" t="inlineStr">
+      <c r="M44" t="inlineStr">
         <is>
           <t>À cadrer</t>
         </is>
@@ -7090,26 +7978,46 @@
       </c>
       <c r="D45" t="inlineStr">
         <is>
+          <t>Pas commencé</t>
+        </is>
+      </c>
+      <c r="E45" t="inlineStr">
+        <is>
+          <t>Pas commencé</t>
+        </is>
+      </c>
+      <c r="F45" t="inlineStr">
+        <is>
+          <t>Pas commencé</t>
+        </is>
+      </c>
+      <c r="G45" t="inlineStr">
+        <is>
+          <t>Pas commencé</t>
+        </is>
+      </c>
+      <c r="H45" t="inlineStr">
+        <is>
           <t>Faible</t>
         </is>
       </c>
-      <c r="E45" t="inlineStr">
-        <is>
-          <t>DSI</t>
-        </is>
-      </c>
-      <c r="F45" t="inlineStr"/>
-      <c r="G45" t="inlineStr">
+      <c r="I45" t="inlineStr">
+        <is>
+          <t>DSI</t>
+        </is>
+      </c>
+      <c r="J45" t="inlineStr"/>
+      <c r="K45" t="inlineStr">
         <is>
           <t>31/10/2026</t>
         </is>
       </c>
-      <c r="H45" t="inlineStr">
+      <c r="L45" t="inlineStr">
         <is>
           <t>Sécurité</t>
         </is>
       </c>
-      <c r="I45" t="inlineStr">
+      <c r="M45" t="inlineStr">
         <is>
           <t>Confort utilisateur</t>
         </is>

</xml_diff>